<commit_message>
Haftalik veri guncellemesi + Ekip sayfasi guncellendi (Elmas Risk Yonetimi'ne, Seyhan Fon Muduru olarak Fon Yonetimi'ne gecti)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Portföy Yöneticisi Yardımcıları</t>
+          <t>Risk Yönetimi</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -4883,17 +4883,17 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Fon Operasyon</t>
+          <t>Fon Yönetimi</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Fon Operasyon</t>
+          <t>Fon Müdürü</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Niyazi Takmaz</t>
+          <t>Seyhan Dönmezkuş</t>
         </is>
       </c>
       <c r="D12" s="8" t="n"/>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Güney Özütutar</t>
+          <t>Niyazi Takmaz</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Aslı Serin</t>
+          <t>Güney Özütutar</t>
         </is>
       </c>
       <c r="D14" s="8" t="n"/>
@@ -4942,12 +4942,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Risk Yönetimi</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Seyhan Dönmezkuş</t>
+          <t>Aslı Serin</t>
         </is>
       </c>
       <c r="D15" s="8" t="n"/>

</xml_diff>

<commit_message>
Haftalik veri guncellemesi + Fon Muduru Fon Operasyon kartina tasindi
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>14229</v>
+        <v>14405</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>48.28</v>
+        <v>48.47</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>56.11</v>
+        <v>56.23</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7712</v>
+        <v>7748</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6369</v>
+        <v>6413</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -3036,7 +3036,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>218.68</v>
+        <v>221.51</v>
       </c>
     </row>
     <row r="6">
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -4883,7 +4883,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Fon Yönetimi</t>
+          <t>Fon Operasyon</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21.5</v>
+        <v>33.7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>18.7</v>
+        <v>29.4</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>30.9</v>
+        <v>42.7</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>40.2</v>
+        <v>53.3</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>26.4</v>
+        <v>40.8</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>33.4</v>
+        <v>51.2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>37.9</v>
+        <v>48.1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46.9</v>
+        <v>46.8</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>36.2</v>
+        <v>37</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>59.4</v>
+        <v>60.1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>24.7</v>
+        <v>26.6</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>39.6</v>
+        <v>41.5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>49.3</v>
+        <v>37.6</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40.1</v>
+        <v>37.6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22.3</v>
+        <v>21.8</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>23.9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15.4</v>
+        <v>19.1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>34.4</v>
+        <v>38.4</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>27.1</v>
+        <v>23.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18.2</v>
+        <v>17.3</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>32.4</v>
+        <v>31.9</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>40.9</v>
+        <v>43.2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25.9</v>
+        <v>30</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31.9</v>
+        <v>38.1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>32.9</v>
+        <v>35.5</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29</v>
+        <v>29.9</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10.3</v>
+        <v>8.1</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>24.8</v>
+        <v>24</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>12.6</v>
+        <v>13</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>30.9</v>
+        <v>31.8</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>25.7</v>
+        <v>26.6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6805,16 +6805,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="E2" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6831,13 +6831,13 @@
         <v>8.300000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6851,16 +6851,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18.2</v>
+        <v>18.3</v>
       </c>
       <c r="E4" t="n">
-        <v>20.9</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6877,13 +6877,13 @@
         <v>43.6</v>
       </c>
       <c r="E5" t="n">
-        <v>45.5</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6897,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>25.7</v>
+        <v>26.6</v>
       </c>
       <c r="E6" t="n">
-        <v>28.1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6920,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="E7" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6943,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8.4</v>
+        <v>11.7</v>
       </c>
       <c r="E8" t="n">
-        <v>2.5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6966,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>12.8</v>
+        <v>13.3</v>
       </c>
       <c r="E9" t="n">
-        <v>9.6</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6989,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>37.9</v>
+        <v>48.1</v>
       </c>
       <c r="E10" t="n">
-        <v>26.4</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7012,16 +7012,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>32.9</v>
+        <v>35.5</v>
       </c>
       <c r="E11" t="n">
-        <v>25.9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7035,16 +7035,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="E12" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7058,7 +7058,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="E13" t="n">
         <v>7.7</v>
@@ -7067,7 +7067,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7081,7 +7081,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15.3</v>
+        <v>14.8</v>
       </c>
       <c r="E14" t="n">
         <v>14.2</v>
@@ -7090,7 +7090,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7104,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>36.2</v>
+        <v>37</v>
       </c>
       <c r="E15" t="n">
-        <v>37.7</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7127,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>32.4</v>
+        <v>31.9</v>
       </c>
       <c r="E16" t="n">
-        <v>33.4</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7150,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="E17" t="n">
-        <v>-7.5</v>
+        <v>-16.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7173,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>-1.3</v>
+        <v>0.2</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7196,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>42.8</v>
+        <v>37.3</v>
       </c>
       <c r="E19" t="n">
-        <v>33.4</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7219,16 +7219,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>59.4</v>
+        <v>60.1</v>
       </c>
       <c r="E20" t="n">
-        <v>39.9</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7242,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>40.9</v>
+        <v>43.2</v>
       </c>
       <c r="E21" t="n">
-        <v>40.3</v>
+        <v>30.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7265,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-3.8</v>
+        <v>-6.9</v>
       </c>
       <c r="E22" t="n">
-        <v>-8.9</v>
+        <v>-14.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7288,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>4.2</v>
+        <v>2.4</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.2</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7311,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3.5</v>
+        <v>2.3</v>
       </c>
       <c r="E24" t="n">
-        <v>9.300000000000001</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7334,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>24.7</v>
+        <v>26.6</v>
       </c>
       <c r="E25" t="n">
-        <v>31.1</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7357,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>18.2</v>
+        <v>17.3</v>
       </c>
       <c r="E26" t="n">
-        <v>28.8</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7380,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>5.9</v>
+        <v>-1.8</v>
       </c>
       <c r="E27" t="n">
-        <v>5.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7403,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1.1</v>
+        <v>3.5</v>
       </c>
       <c r="E28" t="n">
-        <v>0.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>9.800000000000001</v>
+        <v>2.5</v>
       </c>
       <c r="E29" t="n">
-        <v>2.6</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7449,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>39.6</v>
+        <v>41.5</v>
       </c>
       <c r="E30" t="n">
-        <v>32.3</v>
+        <v>30.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7472,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>27.1</v>
+        <v>23.5</v>
       </c>
       <c r="E31" t="n">
-        <v>19.9</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7495,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>-0.5</v>
+        <v>2.1</v>
       </c>
       <c r="E32" t="n">
-        <v>4.8</v>
+        <v>8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7518,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1.5</v>
+        <v>4.6</v>
       </c>
       <c r="E33" t="n">
-        <v>9.5</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>3.3</v>
       </c>
       <c r="E34" t="n">
-        <v>14.4</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7564,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>18.7</v>
+        <v>29.4</v>
       </c>
       <c r="E35" t="n">
-        <v>33.4</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7587,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>15.4</v>
+        <v>19.1</v>
       </c>
       <c r="E36" t="n">
-        <v>31.9</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7610,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4623.4</v>
+        <v>4776.8</v>
       </c>
       <c r="E37" t="n">
-        <v>5256.7</v>
+        <v>5508.1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7633,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2.4</v>
+        <v>4.9</v>
       </c>
       <c r="E38" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4.1</v>
+        <v>5.9</v>
       </c>
       <c r="E39" t="n">
-        <v>2.5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7679,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>6.7</v>
+        <v>8.5</v>
       </c>
       <c r="E40" t="n">
-        <v>9.6</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7702,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21.5</v>
+        <v>33.7</v>
       </c>
       <c r="E41" t="n">
-        <v>26.4</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7725,16 +7725,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>23.9</v>
       </c>
       <c r="E42" t="n">
-        <v>25.9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7748,16 +7748,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6142.4</v>
+        <v>6343.6</v>
       </c>
       <c r="E43" t="n">
-        <v>2709.1</v>
+        <v>2800.3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7771,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>83.40000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="E44" t="n">
-        <v>81.3</v>
+        <v>88.90000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7794,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1232.3</v>
+        <v>1290.4</v>
       </c>
       <c r="E45" t="n">
-        <v>978.7</v>
+        <v>1036.9</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7817,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1.5</v>
+        <v>2.7</v>
       </c>
       <c r="E46" t="n">
-        <v>2.7</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7840,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2.2</v>
+        <v>6.2</v>
       </c>
       <c r="E47" t="n">
-        <v>6.8</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7866,13 +7866,13 @@
         <v>21.9</v>
       </c>
       <c r="E48" t="n">
-        <v>27.4</v>
+        <v>25.4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>40.2</v>
+        <v>53.3</v>
       </c>
       <c r="E49" t="n">
-        <v>46.9</v>
+        <v>58.4</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7909,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>34.4</v>
+        <v>38.4</v>
       </c>
       <c r="E50" t="n">
-        <v>45.8</v>
+        <v>49.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7932,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>8.199999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="E51" t="n">
-        <v>7.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7955,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>4.2</v>
+        <v>7.5</v>
       </c>
       <c r="E52" t="n">
-        <v>5.1</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7978,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.5</v>
       </c>
       <c r="E53" t="n">
-        <v>-5.9</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8001,16 +8001,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>49.3</v>
+        <v>37.6</v>
       </c>
       <c r="E54" t="n">
-        <v>51.7</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8024,16 +8024,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>10.3</v>
+        <v>8.1</v>
       </c>
       <c r="E55" t="n">
-        <v>13.9</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8047,13 +8047,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8067,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>7.9</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8087,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>23.2</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8107,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>40.1</v>
+        <v>37.6</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8127,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>24.8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8147,7 +8147,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="E61" t="n">
         <v>3.4</v>
@@ -8156,7 +8156,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8173,13 +8173,13 @@
         <v>10.5</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8202,7 +8202,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8216,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>49.8</v>
+        <v>49.7</v>
       </c>
       <c r="E64" t="n">
-        <v>46.9</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8239,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>30.9</v>
+        <v>31.8</v>
       </c>
       <c r="E65" t="n">
-        <v>29</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="E66" t="n">
         <v>0.2</v>
@@ -8271,7 +8271,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>6.2</v>
+        <v>5.4</v>
       </c>
       <c r="E67" t="n">
         <v>0.6</v>
@@ -8294,7 +8294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="E68" t="n">
         <v>1.2</v>
@@ -8317,7 +8317,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>22.3</v>
+        <v>21.8</v>
       </c>
       <c r="E69" t="n">
         <v>2.1</v>
@@ -8340,7 +8340,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8354,16 +8354,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="E70" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8383,7 +8383,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8403,7 +8403,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8480,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8505,7 +8505,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8530,7 +8530,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8549,13 +8549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.9</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8574,13 +8574,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8599,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>12.6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8630,7 +8630,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8649,13 +8649,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8680,7 +8680,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8699,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>46.9</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8724,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8749,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>9.9</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8774,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>13.3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>14.4</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8824,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>42.2</v>
+        <v>40.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8849,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>37.2</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-6.1</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8899,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>-2.7</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>13.9</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8949,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>29.5</v>
+        <v>41.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8974,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>26.3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8999,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>2.5</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9024,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>10.4</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9049,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>30.6</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9074,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>36.5</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9099,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>27.8</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9124,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-26.1</v>
+        <v>-42.6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9149,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>-7.9</v>
+        <v>-22.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9174,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>38.5</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9199,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>46.2</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9224,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>63.4</v>
+        <v>41.4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.4</v>
+        <v>3.36</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9274,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.74</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9305,7 +9305,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9324,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>50.02</v>
+        <v>49.86</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>31.18</v>
+        <v>32.17</v>
       </c>
     </row>
   </sheetData>
@@ -9463,7 +9463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9497,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9511,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9.1</v>
+        <v>9.470000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9531,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.800000000000001</v>
+        <v>8.94</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9551,13 +9551,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.14</v>
+        <v>3.42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9571,13 +9571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4.87</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9591,13 +9591,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.35</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9611,13 +9611,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9631,13 +9631,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.22</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9651,13 +9651,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.93</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9671,13 +9671,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>40.42</v>
+        <v>32.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9691,13 +9691,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.68</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9711,13 +9711,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>25.74</v>
+        <v>31.99</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9731,13 +9731,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9751,13 +9751,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3.65</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9771,13 +9771,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>66.98</v>
+        <v>66.13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9791,13 +9791,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29.37</v>
+        <v>29.52</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9811,13 +9811,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>89.02</v>
+        <v>82.45</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9831,33 +9831,33 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7.35</v>
+        <v>17.55</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AAV</t>
+          <t>AED</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Devlet Tahvili</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3.63</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9867,17 +9867,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Devlet Tahvili</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10.56</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9887,17 +9887,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>3.24</v>
+        <v>53.43</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9907,17 +9907,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>56.7</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9931,13 +9931,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>21.45</v>
+        <v>13.02</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9951,13 +9951,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.050000000000001</v>
+        <v>8.08</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9971,13 +9971,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>90.61</v>
+        <v>90.56999999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9991,13 +9991,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7.42</v>
+        <v>7.47</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10011,13 +10011,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.97</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10031,13 +10031,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>89.22</v>
+        <v>92.55</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10071,13 +10071,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10091,13 +10091,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9.73</v>
+        <v>6.28</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10117,7 +10117,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10131,13 +10131,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7.26</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.59</v>
+        <v>0.65</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10167,17 +10167,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>21.87</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10187,17 +10187,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.18</v>
+        <v>30.99</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -10207,37 +10207,37 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>67.92</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>23.19</v>
+        <v>58.15</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10247,17 +10247,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.02</v>
+        <v>23.98</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10267,17 +10267,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>70.39</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -10287,57 +10287,57 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>6.4</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>8.800000000000001</v>
+        <v>66.69</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>3.4</v>
+        <v>6.71</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10347,17 +10347,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Kıymetli Maden</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>82.42</v>
+        <v>8.98</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10367,97 +10367,97 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Kamu Kira Sertifikası (TL)</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>5.38</v>
+        <v>3.52</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Kıymetli Maden</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>83.11</v>
+        <v>82.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>16.89</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>19.67</v>
+        <v>83.91</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.19</v>
+        <v>16.09</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10467,17 +10467,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>67.59</v>
+        <v>19.52</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10487,42 +10487,42 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>12.55</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>89.43000000000001</v>
+        <v>65.67</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -10531,53 +10531,53 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>10.57</v>
+        <v>12.82</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1.54</v>
+        <v>87.15000000000001</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>16.1</v>
+        <v>12.85</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10587,17 +10587,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>3.32</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10607,17 +10607,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.02</v>
+        <v>17.96</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10627,17 +10627,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>69.59999999999999</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -10647,57 +10647,57 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>9.42</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>28.81</v>
+        <v>68.22</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4.82</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -10707,17 +10707,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>65.86</v>
+        <v>27.56</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -10727,11 +10727,51 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
+          <t>VİOP Teminatı</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>10.22</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Yabancı Hisse Senedi</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>61.73</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
           <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
-      <c r="D63" t="n">
-        <v>0.51</v>
+      <c r="D65" t="n">
+        <v>0.49</v>
       </c>
     </row>
   </sheetData>
@@ -10841,25 +10881,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21.5</v>
+        <v>33.7</v>
       </c>
       <c r="E2" t="n">
-        <v>83.40000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>1232.3</v>
+        <v>1290.4</v>
       </c>
       <c r="G2" t="n">
-        <v>6142.4</v>
+        <v>6343.6</v>
       </c>
       <c r="H2" t="n">
-        <v>22.4</v>
+        <v>23.7</v>
       </c>
       <c r="I2" t="n">
-        <v>67.8</v>
+        <v>69.3</v>
       </c>
       <c r="J2" t="n">
-        <v>34.9</v>
+        <v>35.2</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10884,25 +10924,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>26.4</v>
+        <v>40.8</v>
       </c>
       <c r="E3" t="n">
-        <v>81.3</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F3" t="n">
-        <v>978.7</v>
+        <v>1036.9</v>
       </c>
       <c r="G3" t="n">
-        <v>2709.1</v>
+        <v>2800.3</v>
       </c>
       <c r="H3" t="n">
-        <v>21.9</v>
+        <v>23.6</v>
       </c>
       <c r="I3" t="n">
-        <v>60.9</v>
+        <v>62.6</v>
       </c>
       <c r="J3" t="n">
-        <v>27.3</v>
+        <v>27.6</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10927,22 +10967,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-4.9</v>
+        <v>-7.1</v>
       </c>
       <c r="E4" t="n">
-        <v>2.1</v>
+        <v>0.5</v>
       </c>
       <c r="F4" t="n">
-        <v>253.6</v>
+        <v>253.5</v>
       </c>
       <c r="G4" t="n">
-        <v>3433.3</v>
+        <v>3543.3</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="I4" t="n">
-        <v>6.9</v>
+        <v>6.7</v>
       </c>
       <c r="J4" t="n">
         <v>7.6</v>
@@ -10970,25 +11010,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24.2</v>
+        <v>36.6</v>
       </c>
       <c r="E5" t="n">
-        <v>93.8</v>
+        <v>100.1</v>
       </c>
       <c r="F5" t="n">
-        <v>1361.2</v>
+        <v>1424.9</v>
       </c>
       <c r="G5" t="n">
-        <v>7830.2</v>
+        <v>8085.8</v>
       </c>
       <c r="H5" t="n">
-        <v>24.7</v>
+        <v>26</v>
       </c>
       <c r="I5" t="n">
-        <v>71</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>37.3</v>
+        <v>37.5</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -11013,25 +11053,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>26.4</v>
+        <v>40.8</v>
       </c>
       <c r="E6" t="n">
-        <v>81.3</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>978.7</v>
+        <v>1036.9</v>
       </c>
       <c r="G6" t="n">
-        <v>2709.1</v>
+        <v>2800.3</v>
       </c>
       <c r="H6" t="n">
-        <v>21.9</v>
+        <v>23.6</v>
       </c>
       <c r="I6" t="n">
-        <v>60.9</v>
+        <v>62.6</v>
       </c>
       <c r="J6" t="n">
-        <v>27.3</v>
+        <v>27.6</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11056,25 +11096,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-2.2</v>
+        <v>-4.2</v>
       </c>
       <c r="E7" t="n">
-        <v>12.5</v>
+        <v>11.2</v>
       </c>
       <c r="F7" t="n">
-        <v>382.5</v>
+        <v>388</v>
       </c>
       <c r="G7" t="n">
-        <v>5121.1</v>
+        <v>5285.5</v>
       </c>
       <c r="H7" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="I7" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J7" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11148,10 +11188,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>22.4</v>
+        <v>23.7</v>
       </c>
       <c r="E2" t="n">
-        <v>21.9</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="3">
@@ -11171,10 +11211,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.6</v>
+        <v>1.7</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="4">
@@ -11194,10 +11234,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.8</v>
+        <v>69.3</v>
       </c>
       <c r="E4" t="n">
-        <v>60.9</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="5">
@@ -11217,10 +11257,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>19.3</v>
       </c>
       <c r="E5" t="n">
-        <v>13.2</v>
+        <v>14.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Haftalik veri guncellemesi + DGH Portfoy Dagilimi grafigini sikistiran hata duzeltildi
DGH'nin 8 kategorili portfoy pastasi legend'i cok uzadiginda
altindaki "Fon vs KYD Mevduat" fiyat grafigine kalan alani
neredeyse sifira indiriyordu (grafik bos gorunuyordu). Kategori
sayisi esigi gectiginde legend satir/yazi boyutu kucultuluyor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Talimatlar" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kapak_Ozet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Fon_Katalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fon_Performans" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fon_Performans_Ek_Kriter" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Fon_Fiyat_Serisi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fon_Portfoy_Dagilimi" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Fon_Getiri_Analizi_Detay" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Fon_Yillik_Getiri_Karsilastirma" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Fon_Temettu_Verimi" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Piyasa_Senaryolari" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Makro_Gostergeler" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Degerleme_CDS_MSCI" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Bist_Yillik_Getiriler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Peer_PE_Karsilastirma" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Fon_Metinleri" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Sabit_Metinler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Fon_Avantajlari_Maddeler" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Vergi_Bireysel_Fon_Listesi" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Vergi_ANZ_Tablosu" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Ekip" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Ekip_Organizasyon" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Ata_Fonlari_Performans_Ozet" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Ata_Fonlari_Performans_Ozet_YBB" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Yatirim_100TL_Dagilim" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Yatirim_100TL_Maddeler" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>14405</v>
+        <v>12291</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>48.47</v>
+        <v>49.01</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>56.23</v>
+        <v>55.13</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7748</v>
+        <v>7743</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6413</v>
+        <v>6320</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -2991,7 +2991,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -3000,13 +3000,13 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>10.81</v>
+        <v>10.13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>15.23</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -3030,13 +3030,13 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>23.2</v>
+        <v>22.69</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>221.51</v>
+        <v>252.1</v>
       </c>
     </row>
     <row r="6">
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -3450,7 +3450,7 @@
     <row r="8">
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
@@ -3459,13 +3459,13 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>19.92</v>
+        <v>18.61</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -3474,13 +3474,13 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>16.92</v>
+        <v>16.41</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
@@ -3489,13 +3489,13 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>14.03</v>
+        <v>14.04</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -3504,13 +3504,13 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>12.37</v>
+        <v>11.86</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -3519,13 +3519,13 @@
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>9.91</v>
+        <v>9.59</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -3534,13 +3534,13 @@
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>9.140000000000001</v>
+        <v>9.630000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -3549,13 +3549,13 @@
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>9.359999999999999</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3564,13 +3564,13 @@
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>9.449999999999999</v>
+        <v>8.66</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3579,13 +3579,13 @@
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>8.34</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -3594,7 +3594,7 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>7.18</v>
+        <v>6.66</v>
       </c>
     </row>
     <row r="18">
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>33.7</v>
+        <v>21</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>29.4</v>
+        <v>12.4</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42.7</v>
+        <v>24</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>53.3</v>
+        <v>33.6</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40.8</v>
+        <v>13.1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>51.2</v>
+        <v>34.2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>48.1</v>
+        <v>31.4</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49.7</v>
+        <v>49.3</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>43.6</v>
+        <v>43.2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46.8</v>
+        <v>46.5</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>37</v>
+        <v>28.8</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>60.1</v>
+        <v>57</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>26.6</v>
+        <v>14</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>41.5</v>
+        <v>11.5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>37.6</v>
+        <v>25.8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>37.6</v>
+        <v>35.6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>21.8</v>
+        <v>18.5</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3.6</v>
+        <v>0.5</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5455,7 +5455,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>34.4</v>
+        <v>29.7</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>23.9</v>
+        <v>16.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>19.1</v>
+        <v>7.9</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>38.4</v>
+        <v>26.7</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>23.5</v>
+        <v>14.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17.3</v>
+        <v>13.5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>31.9</v>
+        <v>22.4</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>43.2</v>
+        <v>48.1</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30</v>
+        <v>10.5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>38.1</v>
+        <v>28.4</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>35.5</v>
+        <v>28</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>29.9</v>
+        <v>32.7</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.8</v>
+        <v>12.1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.7</v>
+        <v>-1.9</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>24</v>
+        <v>26.3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>13</v>
+        <v>14.3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>31.8</v>
+        <v>34.7</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>26.6</v>
+        <v>29.3</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5840,7 +5840,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>24.8</v>
+        <v>24.3</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6805,16 +6805,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="E2" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6828,16 +6828,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>10.4</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6854,13 +6854,13 @@
         <v>18.3</v>
       </c>
       <c r="E4" t="n">
-        <v>21.3</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6874,16 +6874,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43.6</v>
+        <v>43.2</v>
       </c>
       <c r="E5" t="n">
-        <v>45.7</v>
+        <v>45.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6897,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>26.6</v>
+        <v>29.3</v>
       </c>
       <c r="E6" t="n">
-        <v>29</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6920,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3.7</v>
+        <v>-3.4</v>
       </c>
       <c r="E7" t="n">
-        <v>2.6</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6943,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>11.7</v>
+        <v>2.2</v>
       </c>
       <c r="E8" t="n">
-        <v>3.9</v>
+        <v>-14.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6966,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>13.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E9" t="n">
-        <v>11.1</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6989,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>48.1</v>
+        <v>31.4</v>
       </c>
       <c r="E10" t="n">
-        <v>40.8</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7012,16 +7012,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>35.5</v>
+        <v>28</v>
       </c>
       <c r="E11" t="n">
-        <v>30</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7035,16 +7035,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3.4</v>
+        <v>-8.1</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>-11.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7058,16 +7058,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>8.4</v>
+        <v>-1.3</v>
       </c>
       <c r="E13" t="n">
-        <v>7.7</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7081,16 +7081,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>14.8</v>
+        <v>4.6</v>
       </c>
       <c r="E14" t="n">
-        <v>14.2</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7104,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>37</v>
+        <v>28.8</v>
       </c>
       <c r="E15" t="n">
-        <v>40.6</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7127,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>31.9</v>
+        <v>22.4</v>
       </c>
       <c r="E16" t="n">
-        <v>33.7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7150,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1.7</v>
+        <v>7.3</v>
       </c>
       <c r="E17" t="n">
-        <v>-16.3</v>
+        <v>-13.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7173,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.2</v>
+        <v>3.9</v>
       </c>
       <c r="E18" t="n">
-        <v>-1.4</v>
+        <v>-10.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7196,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>37.3</v>
+        <v>50.3</v>
       </c>
       <c r="E19" t="n">
-        <v>24.2</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7219,16 +7219,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>60.1</v>
+        <v>57</v>
       </c>
       <c r="E20" t="n">
-        <v>31.7</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7242,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>43.2</v>
+        <v>48.1</v>
       </c>
       <c r="E21" t="n">
-        <v>30.9</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7265,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-6.9</v>
+        <v>-4.1</v>
       </c>
       <c r="E22" t="n">
-        <v>-14.7</v>
+        <v>-15.1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7288,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>2.4</v>
+        <v>-5.1</v>
       </c>
       <c r="E23" t="n">
-        <v>-5.5</v>
+        <v>-21</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7311,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2.3</v>
+        <v>5.7</v>
       </c>
       <c r="E24" t="n">
-        <v>5.1</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7334,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>26.6</v>
+        <v>14</v>
       </c>
       <c r="E25" t="n">
-        <v>28.4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7357,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>17.3</v>
+        <v>13.5</v>
       </c>
       <c r="E26" t="n">
-        <v>23.8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7380,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-1.8</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>-13.7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7403,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.5</v>
+        <v>-4.8</v>
       </c>
       <c r="E28" t="n">
-        <v>1.9</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2.5</v>
+        <v>1.3</v>
       </c>
       <c r="E29" t="n">
-        <v>-0.6</v>
+        <v>-10.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7449,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>41.5</v>
+        <v>11.5</v>
       </c>
       <c r="E30" t="n">
-        <v>30.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7472,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>23.5</v>
+        <v>14.5</v>
       </c>
       <c r="E31" t="n">
-        <v>17.7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7495,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2.1</v>
+        <v>-6.3</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7518,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4.6</v>
+        <v>-4.6</v>
       </c>
       <c r="E33" t="n">
-        <v>11.7</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>3.3</v>
+        <v>-0.9</v>
       </c>
       <c r="E34" t="n">
-        <v>18.1</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7564,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>29.4</v>
+        <v>12.4</v>
       </c>
       <c r="E35" t="n">
-        <v>51.2</v>
+        <v>34.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7587,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>19.1</v>
+        <v>7.9</v>
       </c>
       <c r="E36" t="n">
-        <v>38.1</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7610,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4776.8</v>
+        <v>4319.3</v>
       </c>
       <c r="E37" t="n">
-        <v>5508.1</v>
+        <v>5111.1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7633,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4.9</v>
+        <v>-2.7</v>
       </c>
       <c r="E38" t="n">
-        <v>2.6</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5.9</v>
+        <v>-0.9</v>
       </c>
       <c r="E39" t="n">
-        <v>3.9</v>
+        <v>-14.7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7679,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8.5</v>
+        <v>5.6</v>
       </c>
       <c r="E40" t="n">
-        <v>11.1</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7702,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>33.7</v>
+        <v>21</v>
       </c>
       <c r="E41" t="n">
-        <v>40.8</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7725,16 +7725,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>23.9</v>
+        <v>16.5</v>
       </c>
       <c r="E42" t="n">
-        <v>30</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7748,16 +7748,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6343.6</v>
+        <v>5958.8</v>
       </c>
       <c r="E43" t="n">
-        <v>2800.3</v>
+        <v>2364.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7771,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>89.40000000000001</v>
+        <v>63</v>
       </c>
       <c r="E44" t="n">
-        <v>88.90000000000001</v>
+        <v>53.4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7794,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1290.4</v>
+        <v>1227.6</v>
       </c>
       <c r="E45" t="n">
-        <v>1036.9</v>
+        <v>891</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7817,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2.7</v>
+        <v>-7.1</v>
       </c>
       <c r="E46" t="n">
-        <v>2.2</v>
+        <v>-20.8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7840,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6.2</v>
+        <v>-2.3</v>
       </c>
       <c r="E47" t="n">
-        <v>9.4</v>
+        <v>-14.8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7863,16 +7863,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>21.9</v>
+        <v>13.5</v>
       </c>
       <c r="E48" t="n">
-        <v>25.4</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>53.3</v>
+        <v>33.6</v>
       </c>
       <c r="E49" t="n">
-        <v>58.4</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7909,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>38.4</v>
+        <v>26.7</v>
       </c>
       <c r="E50" t="n">
-        <v>49.2</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7932,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.3</v>
+        <v>-0.8</v>
       </c>
       <c r="E51" t="n">
-        <v>0.7</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7955,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="E52" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7978,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-7.5</v>
+        <v>-0.1</v>
       </c>
       <c r="E53" t="n">
-        <v>-5.4</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8001,16 +8001,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>37.6</v>
+        <v>25.8</v>
       </c>
       <c r="E54" t="n">
-        <v>40.8</v>
+        <v>30.2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8024,16 +8024,16 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>8.1</v>
+        <v>6</v>
       </c>
       <c r="E55" t="n">
-        <v>11.9</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8047,13 +8047,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8067,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8.9</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8087,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>21.9</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8107,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>37.6</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8127,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>24</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8147,16 +8147,16 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="E61" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8170,16 +8170,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10.5</v>
+        <v>10.2</v>
       </c>
       <c r="E62" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>22.8</v>
+        <v>22.6</v>
       </c>
       <c r="E63" t="n">
         <v>21.4</v>
@@ -8202,7 +8202,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8216,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>49.7</v>
+        <v>49.3</v>
       </c>
       <c r="E64" t="n">
-        <v>46.8</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8239,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>31.8</v>
+        <v>34.7</v>
       </c>
       <c r="E65" t="n">
-        <v>29.9</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1</v>
+        <v>-1.6</v>
       </c>
       <c r="E66" t="n">
         <v>0.2</v>
@@ -8271,7 +8271,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8285,16 +8285,16 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>5.4</v>
+        <v>1.9</v>
       </c>
       <c r="E67" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8308,16 +8308,16 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8331,16 +8331,16 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>21.8</v>
+        <v>18.5</v>
       </c>
       <c r="E69" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8354,16 +8354,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>13.8</v>
+        <v>12.1</v>
       </c>
       <c r="E70" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8377,13 +8377,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8397,13 +8397,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10.3</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
     </row>
   </sheetData>
@@ -8480,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8505,7 +8505,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8524,13 +8524,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8549,13 +8549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10.1</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8574,13 +8574,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8599,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8624,13 +8624,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8649,13 +8649,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8680,7 +8680,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8699,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>46.8</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8724,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29.9</v>
+        <v>32.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8749,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>7.9</v>
+        <v>-6.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8774,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>15.5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8824,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>40.1</v>
+        <v>33.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8849,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>36.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-3.4</v>
+        <v>-20</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8899,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>-2</v>
+        <v>-26.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>11.7</v>
+        <v>-10.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8949,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>41.5</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8974,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>29</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8999,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>-2.1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9024,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>9.699999999999999</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9049,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>28.5</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9074,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>31.9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9099,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>25.3</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9124,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-42.6</v>
+        <v>-47.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9149,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>-22.2</v>
+        <v>-51.3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9174,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>16.1</v>
+        <v>-30.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9199,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>31.3</v>
+        <v>-16</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9224,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>41.4</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.36</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9274,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.7</v>
+        <v>10.51</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9299,13 +9299,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.6</v>
+        <v>22.45</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9324,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>49.86</v>
+        <v>49.37</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>32.17</v>
+        <v>35.08</v>
       </c>
     </row>
   </sheetData>
@@ -9463,7 +9463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9497,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9511,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9.470000000000001</v>
+        <v>10.05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9531,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.94</v>
+        <v>8.82</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9551,13 +9551,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.42</v>
+        <v>3.82</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9571,13 +9571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>6.35</v>
+        <v>7.13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9587,17 +9587,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.21</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9607,17 +9607,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.78</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9627,17 +9627,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.33</v>
+        <v>16.59</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9647,17 +9647,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Takasbank Para Piyasası</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1.3</v>
+        <v>22.85</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9667,17 +9667,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>32.25</v>
+        <v>2.76</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9687,17 +9687,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2.92</v>
+        <v>25.79</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9707,22 +9707,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>31.99</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AAL</t>
+          <t>AAS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9731,13 +9731,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.04</v>
+        <v>11.46</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9747,17 +9747,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4.35</v>
+        <v>72.03</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9767,37 +9767,37 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>66.13</v>
+        <v>16.51</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AAS</t>
+          <t>AAV</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>29.52</v>
+        <v>85.88</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9807,17 +9807,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>82.45</v>
+        <v>5.61</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9831,13 +9831,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>17.55</v>
+        <v>8.51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9851,13 +9851,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.47</v>
+        <v>9.18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9871,13 +9871,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3.2</v>
+        <v>4.13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9891,13 +9891,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>53.43</v>
+        <v>60.76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9907,22 +9907,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>21.8</v>
+        <v>25.93</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -9931,93 +9931,93 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>13.02</v>
+        <v>6.13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Özel Sektör Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>8.08</v>
+        <v>93.87</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Kamu Dış Borçlanma Araçları</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>90.56999999999999</v>
+        <v>87.17</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (Döviz)</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7.47</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ANZ</t>
+          <t>AYA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1.96</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10027,17 +10027,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>92.55</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10047,57 +10047,57 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>5.93</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.17</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6.28</v>
+        <v>11.37</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10107,17 +10107,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10127,17 +10127,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7.3</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.65</v>
+        <v>16.59</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10167,17 +10167,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.55</v>
+        <v>29.63</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10187,17 +10187,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>30.99</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -10207,37 +10207,37 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.18</v>
+        <v>38.15</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>58.15</v>
+        <v>22.56</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10247,17 +10247,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>23.98</v>
+        <v>69.03</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10267,77 +10267,77 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2.46</v>
+        <v>8.41</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.16</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>66.69</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Kıymetli Maden</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>6.71</v>
+        <v>82.31</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10347,117 +10347,117 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8.98</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Kamu Kira Sertifikası (TL)</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3.52</v>
+        <v>76.06</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Kıymetli Maden</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>82.8</v>
+        <v>23.94</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>4.7</v>
+        <v>18.14</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>83.91</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>16.09</v>
+        <v>69.41</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10467,82 +10467,82 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>19.52</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>1.99</v>
+        <v>87.55</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>65.67</v>
+        <v>12.45</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>12.82</v>
+        <v>2.17</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -10551,33 +10551,33 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>87.15000000000001</v>
+        <v>14.41</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>12.85</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10587,17 +10587,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.68</v>
+        <v>67.91</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10607,42 +10607,42 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>17.96</v>
+        <v>12.85</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>YLC</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.63</v>
+        <v>27.75</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>YLC</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -10651,18 +10651,18 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.11</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>YLC</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -10671,18 +10671,18 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>68.22</v>
+        <v>67.54000000000001</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>YLC</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -10691,87 +10691,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>10.4</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>YLC</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Yerli Hisse Senedi</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>27.56</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>YLC</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>VİOP Teminatı</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>10.22</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>YLC</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Yabancı Hisse Senedi</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>61.73</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>YLC</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Yatırım Fonu Katılma Payı</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -10881,25 +10801,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>33.7</v>
+        <v>21</v>
       </c>
       <c r="E2" t="n">
-        <v>89.40000000000001</v>
+        <v>63</v>
       </c>
       <c r="F2" t="n">
-        <v>1290.4</v>
+        <v>1227.6</v>
       </c>
       <c r="G2" t="n">
-        <v>6343.6</v>
+        <v>5958.8</v>
       </c>
       <c r="H2" t="n">
-        <v>23.7</v>
+        <v>17.7</v>
       </c>
       <c r="I2" t="n">
-        <v>69.3</v>
+        <v>67.7</v>
       </c>
       <c r="J2" t="n">
-        <v>35.2</v>
+        <v>34.4</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10924,25 +10844,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>40.8</v>
+        <v>13.1</v>
       </c>
       <c r="E3" t="n">
-        <v>88.90000000000001</v>
+        <v>53.4</v>
       </c>
       <c r="F3" t="n">
-        <v>1036.9</v>
+        <v>891</v>
       </c>
       <c r="G3" t="n">
-        <v>2800.3</v>
+        <v>2364.5</v>
       </c>
       <c r="H3" t="n">
-        <v>23.6</v>
+        <v>15.3</v>
       </c>
       <c r="I3" t="n">
-        <v>62.6</v>
+        <v>58.2</v>
       </c>
       <c r="J3" t="n">
-        <v>27.6</v>
+        <v>26</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10967,25 +10887,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-7.1</v>
+        <v>7.9</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5</v>
+        <v>9.6</v>
       </c>
       <c r="F4" t="n">
-        <v>253.5</v>
+        <v>336.6</v>
       </c>
       <c r="G4" t="n">
-        <v>3543.3</v>
+        <v>3594.3</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1</v>
+        <v>2.4</v>
       </c>
       <c r="I4" t="n">
-        <v>6.7</v>
+        <v>9.5</v>
       </c>
       <c r="J4" t="n">
-        <v>7.6</v>
+        <v>8.4</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -11010,25 +10930,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>36.6</v>
+        <v>23.7</v>
       </c>
       <c r="E5" t="n">
-        <v>100.1</v>
+        <v>72.2</v>
       </c>
       <c r="F5" t="n">
-        <v>1424.9</v>
+        <v>1356.1</v>
       </c>
       <c r="G5" t="n">
-        <v>8085.8</v>
+        <v>7597</v>
       </c>
       <c r="H5" t="n">
-        <v>26</v>
+        <v>19.9</v>
       </c>
       <c r="I5" t="n">
-        <v>72.40000000000001</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="J5" t="n">
-        <v>37.5</v>
+        <v>36.7</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -11053,25 +10973,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40.8</v>
+        <v>13.1</v>
       </c>
       <c r="E6" t="n">
-        <v>88.90000000000001</v>
+        <v>53.4</v>
       </c>
       <c r="F6" t="n">
-        <v>1036.9</v>
+        <v>891</v>
       </c>
       <c r="G6" t="n">
-        <v>2800.3</v>
+        <v>2364.5</v>
       </c>
       <c r="H6" t="n">
-        <v>23.6</v>
+        <v>15.3</v>
       </c>
       <c r="I6" t="n">
-        <v>62.6</v>
+        <v>58.2</v>
       </c>
       <c r="J6" t="n">
-        <v>27.6</v>
+        <v>26</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11096,25 +11016,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-4.2</v>
+        <v>10.6</v>
       </c>
       <c r="E7" t="n">
-        <v>11.2</v>
+        <v>18.8</v>
       </c>
       <c r="F7" t="n">
-        <v>388</v>
+        <v>465.1</v>
       </c>
       <c r="G7" t="n">
-        <v>5285.5</v>
+        <v>5232.5</v>
       </c>
       <c r="H7" t="n">
-        <v>2.4</v>
+        <v>4.6</v>
       </c>
       <c r="I7" t="n">
-        <v>9.800000000000001</v>
+        <v>12.7</v>
       </c>
       <c r="J7" t="n">
-        <v>9.9</v>
+        <v>10.7</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11188,10 +11108,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>23.7</v>
+        <v>17.7</v>
       </c>
       <c r="E2" t="n">
-        <v>23.6</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="3">
@@ -11211,10 +11131,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.7</v>
+        <v>-3</v>
       </c>
       <c r="E3" t="n">
-        <v>1.6</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="4">
@@ -11234,10 +11154,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>69.3</v>
+        <v>67.7</v>
       </c>
       <c r="E4" t="n">
-        <v>62.6</v>
+        <v>58.2</v>
       </c>
     </row>
     <row r="5">
@@ -11257,10 +11177,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19.3</v>
+        <v>19.1</v>
       </c>
       <c r="E5" t="n">
-        <v>14.6</v>
+        <v>12.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AYA temettu verimi tablosuna 2026 Ekim (%0,75) eklendi, 2023 Temmuz cikarildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1198,11 +1198,11 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>2023 Temmuz</t>
+          <t>2024 Ocak</t>
         </is>
       </c>
       <c r="D2" s="8" t="n">
-        <v>8.33</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="3">
@@ -1216,11 +1216,11 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>2024 Ocak</t>
+          <t>2024 Nisan</t>
         </is>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1.16</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="4">
@@ -1234,11 +1234,11 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>2024 Nisan</t>
+          <t>2024 Temmuz</t>
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1.09</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="5">
@@ -1252,11 +1252,11 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>2024 Temmuz</t>
+          <t>2024 Ekim</t>
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>3.32</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="6">
@@ -1270,11 +1270,11 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>2024 Ekim</t>
+          <t>2025 Ocak</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1.94</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="7">
@@ -1288,11 +1288,11 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>2025 Ocak</t>
+          <t>2025 Nisan</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.99</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="8">
@@ -1306,11 +1306,11 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>2025 Nisan</t>
+          <t>2025 Temmuz</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>2.52</v>
+        <v>5.03</v>
       </c>
     </row>
     <row r="9">
@@ -1324,11 +1324,11 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>2025 Temmuz</t>
+          <t>2025 Ekim</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>5.03</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="10">
@@ -1342,11 +1342,11 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>2025 Ekim</t>
+          <t>2026 Ocak</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0.76</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="11">
@@ -1360,11 +1360,11 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>2026 Ocak</t>
+          <t>2026 Nisan</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0.59</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="12">
@@ -1378,11 +1378,11 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>2026 Nisan</t>
+          <t>2026 Temmuz</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1.83</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="13">
@@ -1396,11 +1396,11 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>2026 Temmuz</t>
+          <t>2026 Ekim</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>1.47</v>
+        <v>0.75</v>
       </c>
     </row>
   </sheetData>
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>12291</v>
+        <v>12374</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>13000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>49.01</v>
+        <v>49.17</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>54.7</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>55.13</v>
+        <v>55.16</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>63.4</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7743</v>
+        <v>7723</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6320</v>
+        <v>6272</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -3036,7 +3036,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>252.1</v>
+        <v>247.8</v>
       </c>
     </row>
     <row r="6">
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>21</v>
+        <v>22.6</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12.4</v>
+        <v>15</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>24</v>
+        <v>26.9</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>33.6</v>
+        <v>32.9</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.1</v>
+        <v>16.2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>34.2</v>
+        <v>37</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>31.4</v>
+        <v>30.6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>43.2</v>
+        <v>43</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28.8</v>
+        <v>28.2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>57</v>
+        <v>52.5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>14</v>
+        <v>12.2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>11.5</v>
+        <v>7</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>25.8</v>
+        <v>19.9</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>35.6</v>
+        <v>34.1</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>18.5</v>
+        <v>19.9</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.5</v>
+        <v>1.6</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>16.5</v>
+        <v>16.9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7.9</v>
+        <v>8.4</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26.7</v>
+        <v>25.3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>14.5</v>
+        <v>13.4</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22.4</v>
+        <v>22.9</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>48.1</v>
+        <v>45.8</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>28.4</v>
+        <v>29.2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>28</v>
+        <v>27.6</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>32.7</v>
+        <v>33.6</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.1</v>
+        <v>13.1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-1.9</v>
+        <v>-1.4</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.3</v>
+        <v>26.6</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.3</v>
+        <v>14.7</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>34.7</v>
+        <v>35.6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>29.3</v>
+        <v>30.2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6808,13 +6808,13 @@
         <v>3.2</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6828,16 +6828,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6851,16 +6851,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18.3</v>
+        <v>18.2</v>
       </c>
       <c r="E4" t="n">
-        <v>21.8</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6874,7 +6874,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43.2</v>
+        <v>43</v>
       </c>
       <c r="E5" t="n">
         <v>45.2</v>
@@ -6883,7 +6883,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6897,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29.3</v>
+        <v>30.2</v>
       </c>
       <c r="E6" t="n">
-        <v>31.6</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6920,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-3.4</v>
+        <v>-5.9</v>
       </c>
       <c r="E7" t="n">
-        <v>-12.5</v>
+        <v>-15.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6943,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.2</v>
+        <v>1.3</v>
       </c>
       <c r="E8" t="n">
-        <v>-14.7</v>
+        <v>-14.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6966,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9.699999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>-3.3</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6989,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>31.4</v>
+        <v>30.6</v>
       </c>
       <c r="E10" t="n">
-        <v>13.1</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>28</v>
+        <v>27.6</v>
       </c>
       <c r="E11" t="n">
         <v>10.5</v>
@@ -7021,7 +7021,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7038,13 +7038,13 @@
         <v>-8.1</v>
       </c>
       <c r="E12" t="n">
-        <v>-11.4</v>
+        <v>-11.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7061,13 +7061,13 @@
         <v>-1.3</v>
       </c>
       <c r="E13" t="n">
-        <v>-4.8</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7081,16 +7081,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4.6</v>
+        <v>4.5</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.7</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7104,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>28.8</v>
+        <v>28.2</v>
       </c>
       <c r="E15" t="n">
-        <v>26.4</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7127,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22.4</v>
+        <v>22.9</v>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7150,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7.3</v>
+        <v>0.8</v>
       </c>
       <c r="E17" t="n">
-        <v>-13.6</v>
+        <v>-10.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7173,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3.9</v>
+        <v>2.4</v>
       </c>
       <c r="E18" t="n">
-        <v>-10.1</v>
+        <v>-10.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7196,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>50.3</v>
+        <v>47</v>
       </c>
       <c r="E19" t="n">
-        <v>18.4</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7219,16 +7219,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>57</v>
+        <v>52.5</v>
       </c>
       <c r="E20" t="n">
-        <v>17.1</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7242,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>48.1</v>
+        <v>45.8</v>
       </c>
       <c r="E21" t="n">
-        <v>18.2</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7265,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-4.1</v>
+        <v>-5.6</v>
       </c>
       <c r="E22" t="n">
-        <v>-15.1</v>
+        <v>-14.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7288,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-5.1</v>
+        <v>-2.5</v>
       </c>
       <c r="E23" t="n">
-        <v>-21</v>
+        <v>-19.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7311,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5.7</v>
+        <v>0.2</v>
       </c>
       <c r="E24" t="n">
-        <v>-5.4</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7334,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>14</v>
+        <v>12.2</v>
       </c>
       <c r="E25" t="n">
-        <v>5.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7357,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>13.5</v>
+        <v>12</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7380,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-8.699999999999999</v>
+        <v>-13.5</v>
       </c>
       <c r="E27" t="n">
-        <v>-13.7</v>
+        <v>-17.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7403,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-4.8</v>
+        <v>-4.4</v>
       </c>
       <c r="E28" t="n">
-        <v>-10.6</v>
+        <v>-10.3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.3</v>
+        <v>-1.4</v>
       </c>
       <c r="E29" t="n">
-        <v>-10.4</v>
+        <v>-12.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7449,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>11.5</v>
+        <v>7</v>
       </c>
       <c r="E30" t="n">
-        <v>0.2</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7472,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>14.5</v>
+        <v>13.4</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7495,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>-6.3</v>
+        <v>-9.1</v>
       </c>
       <c r="E32" t="n">
-        <v>-2.1</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7518,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-4.6</v>
+        <v>-4.7</v>
       </c>
       <c r="E33" t="n">
-        <v>4.5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>-0.9</v>
+        <v>-1.2</v>
       </c>
       <c r="E34" t="n">
-        <v>11.6</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7564,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>12.4</v>
+        <v>15</v>
       </c>
       <c r="E35" t="n">
-        <v>34.2</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7587,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>7.9</v>
+        <v>8.4</v>
       </c>
       <c r="E36" t="n">
-        <v>28.4</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7610,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4319.3</v>
+        <v>4336.8</v>
       </c>
       <c r="E37" t="n">
-        <v>5111.1</v>
+        <v>5145.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7633,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-2.7</v>
+        <v>-5.4</v>
       </c>
       <c r="E38" t="n">
-        <v>-12.5</v>
+        <v>-15.2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-0.9</v>
+        <v>-0.1</v>
       </c>
       <c r="E39" t="n">
-        <v>-14.7</v>
+        <v>-14.1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7679,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="E40" t="n">
-        <v>-3.3</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7702,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>21</v>
+        <v>22.6</v>
       </c>
       <c r="E41" t="n">
-        <v>13.1</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7725,7 +7725,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>16.5</v>
+        <v>16.9</v>
       </c>
       <c r="E42" t="n">
         <v>10.5</v>
@@ -7734,7 +7734,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7748,7 +7748,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5958.8</v>
+        <v>5979.8</v>
       </c>
       <c r="E43" t="n">
         <v>2364.5</v>
@@ -7757,7 +7757,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7771,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>63</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="E44" t="n">
-        <v>53.4</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7794,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1227.6</v>
+        <v>1223</v>
       </c>
       <c r="E45" t="n">
-        <v>891</v>
+        <v>893.4</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7817,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>-7.1</v>
+        <v>-9.6</v>
       </c>
       <c r="E46" t="n">
-        <v>-20.8</v>
+        <v>-21.7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7840,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-2.3</v>
+        <v>-3.8</v>
       </c>
       <c r="E47" t="n">
-        <v>-14.8</v>
+        <v>-14.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7863,16 +7863,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>13.5</v>
+        <v>11.1</v>
       </c>
       <c r="E48" t="n">
-        <v>-1.8</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>33.6</v>
+        <v>32.9</v>
       </c>
       <c r="E49" t="n">
-        <v>16.2</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7909,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>26.7</v>
+        <v>25.3</v>
       </c>
       <c r="E50" t="n">
-        <v>17.7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7932,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>-0.8</v>
+        <v>-3</v>
       </c>
       <c r="E51" t="n">
-        <v>-0.3</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7955,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5.5</v>
+        <v>6.9</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7978,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-0.1</v>
+        <v>-2</v>
       </c>
       <c r="E53" t="n">
-        <v>2.2</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8001,16 +8001,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>25.8</v>
+        <v>19.9</v>
       </c>
       <c r="E54" t="n">
-        <v>30.2</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8027,13 +8027,13 @@
         <v>6</v>
       </c>
       <c r="E55" t="n">
-        <v>10.1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8047,13 +8047,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8067,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>9.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8087,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>28.8</v>
+        <v>26.8</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8107,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>35.6</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8127,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>26.3</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8150,13 +8150,13 @@
         <v>3.3</v>
       </c>
       <c r="E61" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8170,16 +8170,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
       <c r="E62" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8196,13 +8196,13 @@
         <v>22.6</v>
       </c>
       <c r="E63" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8216,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>49.3</v>
+        <v>49.2</v>
       </c>
       <c r="E64" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8239,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>34.7</v>
+        <v>35.6</v>
       </c>
       <c r="E65" t="n">
-        <v>32.7</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8262,16 +8262,16 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>-1.6</v>
+        <v>-0.9</v>
       </c>
       <c r="E66" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1.9</v>
+        <v>2.4</v>
       </c>
       <c r="E67" t="n">
         <v>0.7</v>
@@ -8294,7 +8294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>10</v>
+        <v>10.4</v>
       </c>
       <c r="E68" t="n">
         <v>1.3</v>
@@ -8317,7 +8317,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>18.5</v>
+        <v>19.9</v>
       </c>
       <c r="E69" t="n">
         <v>2.2</v>
@@ -8340,7 +8340,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8354,16 +8354,16 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>12.1</v>
+        <v>13.1</v>
       </c>
       <c r="E70" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8377,13 +8377,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8397,13 +8397,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>10.1</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
     </row>
   </sheetData>
@@ -8480,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8499,13 +8499,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8530,7 +8530,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8555,7 +8555,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8580,7 +8580,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8599,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>14.3</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8624,13 +8624,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8649,13 +8649,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>9.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8674,13 +8674,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>21.4</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8699,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8724,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>32.7</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8749,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>-6.8</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8774,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>6.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8824,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>33.9</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8849,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>28.7</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-20</v>
+        <v>-18.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8899,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>-26.5</v>
+        <v>-22.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>-10.9</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8949,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>12.3</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8974,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1.1</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8999,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>4.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9024,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>12.1</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9049,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>44.8</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9074,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>35</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9099,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>32.5</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9124,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-47.5</v>
+        <v>-41.6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9149,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>-51.3</v>
+        <v>-54.3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9174,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>-30.7</v>
+        <v>-33.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9199,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>-16</v>
+        <v>-18.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9224,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>-8.199999999999999</v>
+        <v>-12.6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.2</v>
+        <v>3.15</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9274,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.51</v>
+        <v>10.43</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9299,13 +9299,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.45</v>
+        <v>22.37</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9324,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>49.37</v>
+        <v>49.21</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>35.08</v>
+        <v>36.05</v>
       </c>
     </row>
   </sheetData>
@@ -9463,7 +9463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9497,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9511,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10.05</v>
+        <v>10.18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9531,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.82</v>
+        <v>8.93</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9551,13 +9551,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.82</v>
+        <v>3.87</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9571,13 +9571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7.13</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9591,13 +9591,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9611,13 +9611,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.44</v>
+        <v>0.8100000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9631,13 +9631,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16.59</v>
+        <v>17.25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9651,13 +9651,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>22.85</v>
+        <v>32.16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9671,13 +9671,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2.76</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9691,18 +9691,18 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>25.79</v>
+        <v>24.24</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AAL</t>
+          <t>AAS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9711,13 +9711,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.07000000000000001</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9727,17 +9727,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11.46</v>
+        <v>72.81999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9747,37 +9747,37 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>72.03</v>
+        <v>16.63</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AAS</t>
+          <t>AAV</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16.51</v>
+        <v>88.89</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9787,17 +9787,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>85.88</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9807,37 +9807,37 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5.61</v>
+        <v>7.86</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AAV</t>
+          <t>AED</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Devlet Tahvili</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8.51</v>
+        <v>9.390000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9847,17 +9847,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Devlet Tahvili</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>9.18</v>
+        <v>4.23</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9867,17 +9867,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4.13</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9887,37 +9887,37 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>60.76</v>
+        <v>26.78</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>AED</t>
+          <t>ANZ</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Kamu Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>25.93</v>
+        <v>84.69</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9927,17 +9927,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Vadeli Mevduat (Döviz)</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6.13</v>
+        <v>12.91</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9947,17 +9947,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Özel Sektör Dış Borçlanma Araçları</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>93.87</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9971,13 +9971,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>87.17</v>
+        <v>85.73999999999999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9991,13 +9991,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.36</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10011,13 +10011,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2.59</v>
+        <v>3.83</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10031,13 +10031,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2.95</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5.93</v>
+        <v>5.79</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10071,13 +10071,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10087,17 +10087,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>11.37</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10107,17 +10107,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.2</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10127,17 +10127,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.86</v>
+        <v>17.82</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Takasbank Para Piyasası</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>16.59</v>
+        <v>43.63</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10167,17 +10167,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>29.63</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10187,37 +10187,37 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1.58</v>
+        <v>35.25</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DGH</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>38.15</v>
+        <v>22.45</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10227,17 +10227,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>22.56</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10251,13 +10251,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>69.03</v>
+        <v>68.48999999999999</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10271,13 +10271,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8.41</v>
+        <v>8.57</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -10291,13 +10291,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>9.33</v>
+        <v>9.41</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -10311,13 +10311,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3.95</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10331,13 +10331,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>82.31</v>
+        <v>82.7</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10351,13 +10351,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>4.41</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10367,17 +10367,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>BİST Vadeli İşlem (Satım)</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>76.06</v>
+        <v>53.49</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10387,37 +10387,37 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>23.94</v>
+        <v>24.94</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>18.14</v>
+        <v>21.57</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10427,17 +10427,17 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.05</v>
+        <v>19.17</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10447,17 +10447,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>69.41</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10467,37 +10467,37 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>12.4</v>
+        <v>68.75</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>87.55</v>
+        <v>11.46</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10507,37 +10507,37 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>12.45</v>
+        <v>89.62</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2.17</v>
+        <v>10.38</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10547,17 +10547,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>14.41</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10567,17 +10567,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2.66</v>
+        <v>15.41</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10587,17 +10587,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>67.91</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10607,37 +10607,37 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>12.85</v>
+        <v>68.09999999999999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27.75</v>
+        <v>13.94</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -10647,17 +10647,17 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>4.21</v>
+        <v>29.43</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10667,17 +10667,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>67.54000000000001</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -10687,11 +10687,31 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
+          <t>Yabancı Hisse Senedi</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>68.48999999999999</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
           <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>0.5</v>
+      <c r="D62" t="n">
+        <v>0.51</v>
       </c>
     </row>
   </sheetData>
@@ -10801,22 +10821,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>22.6</v>
       </c>
       <c r="E2" t="n">
-        <v>63</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F2" t="n">
-        <v>1227.6</v>
+        <v>1223</v>
       </c>
       <c r="G2" t="n">
-        <v>5958.8</v>
+        <v>5979.8</v>
       </c>
       <c r="H2" t="n">
-        <v>17.7</v>
+        <v>19.9</v>
       </c>
       <c r="I2" t="n">
-        <v>67.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="J2" t="n">
         <v>34.4</v>
@@ -10844,25 +10864,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>13.1</v>
+        <v>16.2</v>
       </c>
       <c r="E3" t="n">
-        <v>53.4</v>
+        <v>54.7</v>
       </c>
       <c r="F3" t="n">
-        <v>891</v>
+        <v>893.4</v>
       </c>
       <c r="G3" t="n">
         <v>2364.5</v>
       </c>
       <c r="H3" t="n">
-        <v>15.3</v>
+        <v>15.7</v>
       </c>
       <c r="I3" t="n">
-        <v>58.2</v>
+        <v>58.3</v>
       </c>
       <c r="J3" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10887,25 +10907,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>7.9</v>
+        <v>6.4</v>
       </c>
       <c r="E4" t="n">
-        <v>9.6</v>
+        <v>17.7</v>
       </c>
       <c r="F4" t="n">
-        <v>336.6</v>
+        <v>329.6</v>
       </c>
       <c r="G4" t="n">
-        <v>3594.3</v>
+        <v>3615.3</v>
       </c>
       <c r="H4" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="I4" t="n">
-        <v>9.5</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J4" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -10930,22 +10950,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>23.7</v>
+        <v>25.3</v>
       </c>
       <c r="E5" t="n">
-        <v>72.2</v>
+        <v>82.2</v>
       </c>
       <c r="F5" t="n">
-        <v>1356.1</v>
+        <v>1351</v>
       </c>
       <c r="G5" t="n">
-        <v>7597</v>
+        <v>7623.7</v>
       </c>
       <c r="H5" t="n">
-        <v>19.9</v>
+        <v>22.1</v>
       </c>
       <c r="I5" t="n">
-        <v>70.90000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="J5" t="n">
         <v>36.7</v>
@@ -10973,25 +10993,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>13.1</v>
+        <v>16.2</v>
       </c>
       <c r="E6" t="n">
-        <v>53.4</v>
+        <v>54.7</v>
       </c>
       <c r="F6" t="n">
-        <v>891</v>
+        <v>893.4</v>
       </c>
       <c r="G6" t="n">
         <v>2364.5</v>
       </c>
       <c r="H6" t="n">
-        <v>15.3</v>
+        <v>15.7</v>
       </c>
       <c r="I6" t="n">
-        <v>58.2</v>
+        <v>58.3</v>
       </c>
       <c r="J6" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11016,25 +11036,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10.6</v>
+        <v>9.1</v>
       </c>
       <c r="E7" t="n">
-        <v>18.8</v>
+        <v>27.5</v>
       </c>
       <c r="F7" t="n">
-        <v>465.1</v>
+        <v>457.6</v>
       </c>
       <c r="G7" t="n">
-        <v>5232.5</v>
+        <v>5259.2</v>
       </c>
       <c r="H7" t="n">
-        <v>4.6</v>
+        <v>6.4</v>
       </c>
       <c r="I7" t="n">
-        <v>12.7</v>
+        <v>12.4</v>
       </c>
       <c r="J7" t="n">
-        <v>10.7</v>
+        <v>10.8</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -11108,10 +11128,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>17.7</v>
+        <v>19.9</v>
       </c>
       <c r="E2" t="n">
-        <v>15.3</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="3">
@@ -11131,10 +11151,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="E3" t="n">
-        <v>-4.9</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="4">
@@ -11154,10 +11174,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>58.2</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="5">
@@ -11180,7 +11200,7 @@
         <v>19.1</v>
       </c>
       <c r="E5" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AYA temettu verimi: 2025 Ekim (0,77) ve 2026 Nisan (1,84) siteye gore duzeltildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1328,7 +1328,7 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="10">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1.83</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
100 TL dagilimi: Turk hisse %35->%30, TL sabit getiri %40->%45
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -5896,7 +5896,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
@@ -5906,7 +5906,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -5966,7 +5966,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -6005,7 +6005,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sayfa 3-4: fon adlarinin yanina fon kodlari eklendi, etiket alani 290px'e genisletildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -5109,7 +5109,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ata İkinci Hisse Senedi Fonu</t>
+          <t>Ata İkinci Hisse Senedi Fonu (AAV)</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ata Kar Payı Ödeyen Hisse Senedi Fonu</t>
+          <t>Ata Kar Payı Ödeyen Hisse Senedi Fonu (AYA)</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ata Kar Payı Ödeyen Hisse Senedi Fonu (Temettü Dahil)</t>
+          <t>Ata Kar Payı Ödeyen Hisse Senedi Fonu (AYA - Temettü Dahil)</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ata Katılım Hisse Senedi Fonu</t>
+          <t>Ata Katılım Hisse Senedi Fonu (TLZ)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ata Birinci Değişken Fon</t>
+          <t>Ata Birinci Değişken Fon (AED)</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -5235,7 +5235,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ata Para Piyasası Serbest (TL) Fon</t>
+          <t>Ata Para Piyasası Serbest (TL) Fon (DGH)</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ata Para Piyasası Fonu</t>
+          <t>Ata Para Piyasası Fonu (AAL)</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ata Tarım ve Gıda Değişken Fon</t>
+          <t>Ata Tarım ve Gıda Değişken Fon (YLC)</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ata Robotik Teknolojileri Değişken Fon</t>
+          <t>Ata Robotik Teknolojileri Değişken Fon (RTG)</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Ata Havacılık ve Savunma Teknolojileri Değişken Fon</t>
+          <t>Ata Havacılık ve Savunma Teknolojileri Değişken Fon (JET)</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ata Enerji Değişken Fon</t>
+          <t>Ata Enerji Değişken Fon (URA)</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5361,7 +5361,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ata Altın Katılım Fonu</t>
+          <t>Ata Altın Katılım Fonu (PKF)</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ata Fon Sepeti Serbest Fon</t>
+          <t>Ata Fon Sepeti Serbest Fon (AAS)</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ata Dördüncü Serbest (Eurobond) Fon (TL Getiri)</t>
+          <t>Ata Dördüncü Serbest (Eurobond) Fon (ANZ - TL Getiri)</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ata Dördüncü Serbest (Eurobond) Fon (USD Getiri)</t>
+          <t>Ata Dördüncü Serbest (Eurobond) Fon (ANZ - USD Getiri)</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -5512,7 +5512,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>İkinci Hisse Senedi Fonu</t>
+          <t>İkinci Hisse Senedi Fonu (AAV)</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -5530,7 +5530,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kar Payı Ödeyen Hisse Senedi Fonu</t>
+          <t>Kar Payı Ödeyen Hisse Senedi Fonu (AYA)</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -5548,7 +5548,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Katılım Hisse Senedi (TL) Fonu</t>
+          <t>Katılım Hisse Senedi (TL) Fonu (TLZ)</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enerji Değişken Fon</t>
+          <t>Enerji Değişken Fon (URA)</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Havacılık ve Savunma Teknolojileri Fonu</t>
+          <t>Havacılık ve Savunma Teknolojileri Fonu (JET)</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -5602,7 +5602,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tarım ve Gıda Değişken Fon</t>
+          <t>Tarım ve Gıda Değişken Fon (YLC)</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Robotik Teknolojileri Değişken Fon</t>
+          <t>Robotik Teknolojileri Değişken Fon (RTG)</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -5674,7 +5674,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ATA Birinci Değişken Fon</t>
+          <t>ATA Birinci Değişken Fon (AED)</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -5710,7 +5710,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ata Altın Katılım Fonu</t>
+          <t>Ata Altın Katılım Fonu (PKF)</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ATA 4. Serbest (EB) Fon (TL Getiri)</t>
+          <t>ATA 4. Serbest (EB) Fon (ANZ - TL Getiri)</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ATA 4. Serbest (EB) Fon (USD Getiri)</t>
+          <t>ATA 4. Serbest (EB) Fon (ANZ - USD Getiri)</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ATA Fon Sepeti Serbest Fon</t>
+          <t>ATA Fon Sepeti Serbest Fon (AAS)</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -5800,7 +5800,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ata Para Piyasası Serbest (TL) Fon</t>
+          <t>Ata Para Piyasası Serbest (TL) Fon (DGH)</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ata Para Piyasası Fonu</t>
+          <t>Ata Para Piyasası Fonu (AAL)</t>
         </is>
       </c>
       <c r="C19" t="n">

</xml_diff>

<commit_message>
Sayfa 6: BIST 100 senaryolari 11.000 / 13.500 / 15.000 olarak guncellendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1478,13 +1478,13 @@
         <v>12374</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>13000</v>
+        <v>11000</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>17000</v>
+        <v>13500</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>19000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Sayfa 6-7: USD/TL (53,00/51,20/50,00) ve EURO/TL (60,50/57,40/55,80) senaryolari guncellendi, 7. sayfa yil sonu kur tahminleri yeni baza cekildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1502,13 +1502,13 @@
         <v>49.17</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>54.7</v>
+        <v>53</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>51.53</v>
+        <v>51.2</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>49.9</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -1526,13 +1526,13 @@
         <v>55.16</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>63.4</v>
+        <v>60.5</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>59.77</v>
+        <v>57.4</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>57.92</v>
+        <v>55.8</v>
       </c>
     </row>
     <row r="5">
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>1.16</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="26">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>51.53</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="38">
@@ -2246,7 +2246,7 @@
         </is>
       </c>
       <c r="C49" s="8" t="n">
-        <v>59.77</v>
+        <v>57.4</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
Sayfa 7: makro tahminler Ata Yatirim verisiyle guncellendi, 2027T sutunu eklendi; Sayfa 6 USD/TL ve EURO/TL baz senaryolari Ata Yatirim yil sonu tahminine (50,67 / 58,27) cekildi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1505,7 +1505,7 @@
         <v>53</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>51.2</v>
+        <v>50.67</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>50</v>
@@ -1529,7 +1529,7 @@
         <v>60.5</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>57.4</v>
+        <v>58.27</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>55.8</v>
@@ -1600,7 +1600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>7249</v>
+        <v>7434</v>
       </c>
     </row>
     <row r="3">
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>15007</v>
+        <v>15326</v>
       </c>
     </row>
     <row r="4">
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>26276</v>
+        <v>27091</v>
       </c>
     </row>
     <row r="5">
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>39806</v>
+        <v>44587</v>
       </c>
     </row>
     <row r="6">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>62905</v>
+        <v>63241</v>
       </c>
     </row>
     <row r="7">
@@ -1700,25 +1700,25 @@
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>82330</v>
+        <v>84500</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>2021</v>
+        <v>2027</v>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>GSYH (milyar $)</t>
+          <t>GSYH (milyar TL)</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>803</v>
+        <v>114000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
@@ -1726,12 +1726,12 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>906</v>
+        <v>828</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
@@ -1739,12 +1739,12 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>1108</v>
+        <v>925</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
@@ -1752,12 +1752,12 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>1214</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
@@ -1765,12 +1765,12 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>1595</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -1778,38 +1778,38 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>1741</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>GSYH Buyumesi</t>
+          <t>GSYH (milyar $)</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>11</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>GSYH Buyumesi</t>
+          <t>GSYH (milyar $)</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>5.6</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
@@ -1817,12 +1817,12 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
@@ -1830,12 +1830,12 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>3.2</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
@@ -1843,12 +1843,12 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>3.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
@@ -1856,51 +1856,51 @@
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>GSYH Buyumesi</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>1.13</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>GSYH Buyumesi</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>1.07</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>2023</v>
+        <v>2027</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>GSYH Buyumesi</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>1.11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
@@ -1908,12 +1908,12 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>1.04</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
@@ -1921,12 +1921,12 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>1.18</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
@@ -1934,64 +1934,64 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>1.18</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>1.05</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>1.08</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
-        <v>2024</v>
+        <v>2027</v>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>1.08</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
@@ -1999,12 +1999,12 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>1.13</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
@@ -2012,77 +2012,77 @@
         </is>
       </c>
       <c r="C31" s="8" t="n">
-        <v>1.17</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>12.98</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>18.7</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>29.44</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>35.22</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>2025</v>
+        <v>2027</v>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>42.86</v>
+        <v>1.16</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
-        <v>2026</v>
+        <v>2021</v>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
@@ -2090,85 +2090,85 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>51.2</v>
+        <v>12.98</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>8.869999999999999</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>16.57</v>
+        <v>29.44</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>23.71</v>
+        <v>35.22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>32.79</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>39.44</v>
+        <v>50.67</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C43" s="8" t="n">
-        <v>47.28</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="44">
@@ -2177,11 +2177,11 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>14.68</v>
+        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="45">
@@ -2190,11 +2190,11 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C45" s="8" t="n">
-        <v>19.93</v>
+        <v>16.57</v>
       </c>
     </row>
     <row r="46">
@@ -2203,11 +2203,11 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>32.57</v>
+        <v>23.71</v>
       </c>
     </row>
     <row r="47">
@@ -2216,11 +2216,11 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C47" s="8" t="n">
-        <v>36.74</v>
+        <v>32.79</v>
       </c>
     </row>
     <row r="48">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>50.45</v>
+        <v>39.44</v>
       </c>
     </row>
     <row r="49">
@@ -2242,479 +2242,479 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C49" s="8" t="n">
-        <v>57.4</v>
+        <v>46.78</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>2021</v>
+        <v>2027</v>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C50" s="8" t="n">
-        <v>10.45</v>
+        <v>55.99</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C51" s="8" t="n">
-        <v>17.39</v>
+        <v>14.68</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C52" s="8" t="n">
-        <v>25.64</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>35.48</v>
+        <v>32.57</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>44.65</v>
+        <v>36.74</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>55.27</v>
+        <v>50.45</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>79.89</v>
+        <v>58.27</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>97.72</v>
+        <v>71.09999999999999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C58" s="8" t="n">
-        <v>44.22</v>
+        <v>10.45</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C59" s="8" t="n">
-        <v>28.52</v>
+        <v>17.39</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C60" s="8" t="n">
-        <v>27.67</v>
+        <v>25.64</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C61" s="8" t="n">
-        <v>20.71</v>
+        <v>35.48</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>36.08</v>
+        <v>44.65</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C63" s="8" t="n">
-        <v>64.27</v>
+        <v>54.02</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>2023</v>
+        <v>2027</v>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C64" s="8" t="n">
-        <v>64.77</v>
+        <v>64.69</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C65" s="8" t="n">
-        <v>44.38</v>
+        <v>79.89</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C66" s="8" t="n">
-        <v>30.89</v>
+        <v>97.72</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C67" s="8" t="n">
-        <v>27.5</v>
+        <v>44.22</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C68" s="8" t="n">
-        <v>-15</v>
+        <v>28.52</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C69" s="8" t="n">
-        <v>-49</v>
+        <v>27.67</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C70" s="8" t="n">
-        <v>-44</v>
+        <v>29.52</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n">
-        <v>2024</v>
+        <v>2027</v>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C71" s="8" t="n">
-        <v>-10</v>
+        <v>20.37</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C72" s="8" t="n">
-        <v>-24</v>
+        <v>36.08</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C73" s="8" t="n">
-        <v>-27</v>
+        <v>64.27</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>-1.9</v>
+        <v>64.77</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C75" s="8" t="n">
-        <v>-5.4</v>
+        <v>44.38</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C76" s="8" t="n">
-        <v>-4</v>
+        <v>30.89</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C77" s="8" t="n">
-        <v>-0.8</v>
+        <v>29.68</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>2025</v>
+        <v>2027</v>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C78" s="8" t="n">
-        <v>-1.5</v>
+        <v>22.98</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>2026</v>
+        <v>2021</v>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C79" s="8" t="n">
-        <v>-1.8</v>
+        <v>-7.2</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C80" s="8" t="n">
-        <v>225</v>
+        <v>-48.8</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C81" s="8" t="n">
-        <v>254</v>
+        <v>-44</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C82" s="8" t="n">
-        <v>255</v>
+        <v>-9.800000000000001</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C83" s="8" t="n">
-        <v>262</v>
+        <v>-24</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>273</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C85" s="8" t="n">
-        <v>285</v>
+        <v>-41</v>
       </c>
     </row>
     <row r="86">
@@ -2723,11 +2723,11 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C86" s="8" t="n">
-        <v>271</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="87">
@@ -2736,11 +2736,11 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C87" s="8" t="n">
-        <v>364</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="88">
@@ -2749,11 +2749,11 @@
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>362</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="89">
@@ -2762,11 +2762,11 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C89" s="8" t="n">
-        <v>344</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="90">
@@ -2775,11 +2775,11 @@
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>366</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="91">
@@ -2788,167 +2788,388 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C91" s="8" t="n">
-        <v>394</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>2021</v>
+        <v>2027</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>-46</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>-110</v>
+        <v>225</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>-107</v>
+        <v>254</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>-82</v>
+        <v>256</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>-92</v>
+        <v>262</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>-109</v>
+        <v>273</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>Brent Petrol (ABD$/varil)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>71</v>
+        <v>280</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="n">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>Brent Petrol (ABD$/varil)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>99</v>
+        <v>289</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>Brent Petrol (ABD$/varil)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>82</v>
+        <v>271</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>Brent Petrol (ABD$/varil)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>80</v>
+        <v>364</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>Brent Petrol (ABD$/varil)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>69</v>
+        <v>362</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B103" s="8" t="inlineStr">
+        <is>
+          <t>Ithalat (cif, milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="n">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B104" s="8" t="inlineStr">
+        <is>
+          <t>Ithalat (cif, milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C104" s="8" t="n">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="8" t="n">
         <v>2026</v>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B105" s="8" t="inlineStr">
+        <is>
+          <t>Ithalat (cif, milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B106" s="8" t="inlineStr">
+        <is>
+          <t>Ithalat (cif, milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B107" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="n">
+        <v>-46</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B108" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="n">
+        <v>-110</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B109" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="n">
+        <v>-106</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="n">
+        <v>-82</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B111" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="n">
+        <v>-92</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B112" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="n">
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="n">
+        <v>-91</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B114" s="8" t="inlineStr">
         <is>
           <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
-      <c r="C103" s="8" t="n">
-        <v>60</v>
+      <c r="C114" s="8" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="8" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>Brent Petrol (ABD$/varil)</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>Brent Petrol (ABD$/varil)</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="8" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>Brent Petrol (ABD$/varil)</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B118" s="8" t="inlineStr">
+        <is>
+          <t>Brent Petrol (ABD$/varil)</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B119" s="8" t="inlineStr">
+        <is>
+          <t>Brent Petrol (ABD$/varil)</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="8" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B120" s="8" t="inlineStr">
+        <is>
+          <t>Brent Petrol (ABD$/varil)</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="n">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sayfa 7: 2027T sutunu kaldirildi (Etem Bey talebi), baslik tekrar '2026 Piyasa ve Makro Tahminleri'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1600,7 +1600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1705,20 +1705,20 @@
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>2027</v>
+        <v>2021</v>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>GSYH (milyar TL)</t>
+          <t>GSYH (milyar $)</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>114000</v>
+        <v>828</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
@@ -1726,12 +1726,12 @@
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>828</v>
+        <v>925</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
@@ -1739,12 +1739,12 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>925</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
@@ -1752,12 +1752,12 @@
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>1153</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
@@ -1765,12 +1765,12 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>1358</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -1778,38 +1778,38 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>1602</v>
+        <v>1806</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>2026</v>
+        <v>2021</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>GSYH (milyar $)</t>
+          <t>GSYH Buyumesi</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>1806</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
-        <v>2027</v>
+        <v>2022</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>GSYH (milyar $)</t>
+          <t>GSYH Buyumesi</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>2036</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
@@ -1817,12 +1817,12 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
@@ -1830,12 +1830,12 @@
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>5.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
@@ -1843,12 +1843,12 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
@@ -1856,51 +1856,51 @@
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>GSYH Buyumesi</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>3.7</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>GSYH Buyumesi</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>3</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>2027</v>
+        <v>2023</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>GSYH Buyumesi</t>
+          <t>Euro/ABD $ (yil sonu)</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>4</v>
+        <v>1.11</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
@@ -1908,12 +1908,12 @@
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>1.13</v>
+        <v>1.04</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
@@ -1921,12 +1921,12 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>1.07</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
@@ -1934,64 +1934,64 @@
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>1.11</v>
+        <v>1.14</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>1.04</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>1.18</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>1.14</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
-        <v>2027</v>
+        <v>2024</v>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (yil sonu)</t>
+          <t>Euro/ABD $ (ortalama)</t>
         </is>
       </c>
       <c r="C29" s="8" t="n">
-        <v>1.16</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
@@ -1999,12 +1999,12 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>1.18</v>
+        <v>1.13</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
@@ -2012,77 +2012,77 @@
         </is>
       </c>
       <c r="C31" s="8" t="n">
-        <v>1.05</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>1.08</v>
+        <v>12.98</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>1.08</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>1.13</v>
+        <v>29.44</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>1.15</v>
+        <v>35.22</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>2027</v>
+        <v>2025</v>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Euro/ABD $ (ortalama)</t>
+          <t>ABD $/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>1.16</v>
+        <v>42.86</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
@@ -2090,85 +2090,85 @@
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>12.98</v>
+        <v>50.67</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>18.7</v>
+        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>29.44</v>
+        <v>16.57</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>35.22</v>
+        <v>23.71</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>42.86</v>
+        <v>32.79</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>50.67</v>
+        <v>39.44</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (yil sonu)</t>
+          <t>ABD $/TL (ortalama)</t>
         </is>
       </c>
       <c r="C43" s="8" t="n">
-        <v>61.3</v>
+        <v>46.78</v>
       </c>
     </row>
     <row r="44">
@@ -2177,11 +2177,11 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>8.869999999999999</v>
+        <v>14.68</v>
       </c>
     </row>
     <row r="45">
@@ -2190,11 +2190,11 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C45" s="8" t="n">
-        <v>16.57</v>
+        <v>19.93</v>
       </c>
     </row>
     <row r="46">
@@ -2203,11 +2203,11 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>23.71</v>
+        <v>32.57</v>
       </c>
     </row>
     <row r="47">
@@ -2216,11 +2216,11 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C47" s="8" t="n">
-        <v>32.79</v>
+        <v>36.74</v>
       </c>
     </row>
     <row r="48">
@@ -2229,11 +2229,11 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C48" s="8" t="n">
-        <v>39.44</v>
+        <v>50.45</v>
       </c>
     </row>
     <row r="49">
@@ -2242,479 +2242,479 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (yil sonu)</t>
         </is>
       </c>
       <c r="C49" s="8" t="n">
-        <v>46.78</v>
+        <v>58.27</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>2027</v>
+        <v>2021</v>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>ABD $/TL (ortalama)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C50" s="8" t="n">
-        <v>55.99</v>
+        <v>10.45</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C51" s="8" t="n">
-        <v>14.68</v>
+        <v>17.39</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C52" s="8" t="n">
-        <v>19.93</v>
+        <v>25.64</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>32.57</v>
+        <v>35.48</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>36.74</v>
+        <v>44.65</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>Euro/TL (ortalama)</t>
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>50.45</v>
+        <v>54.02</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
-        <v>2026</v>
+        <v>2021</v>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>58.27</v>
+        <v>79.89</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>2027</v>
+        <v>2022</v>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (yil sonu)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>71.09999999999999</v>
+        <v>97.72</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C58" s="8" t="n">
-        <v>10.45</v>
+        <v>44.22</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C59" s="8" t="n">
-        <v>17.39</v>
+        <v>28.52</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C60" s="8" t="n">
-        <v>25.64</v>
+        <v>27.67</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>UFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C61" s="8" t="n">
-        <v>35.48</v>
+        <v>29.52</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>2025</v>
+        <v>2021</v>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>44.65</v>
+        <v>36.08</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>2026</v>
+        <v>2022</v>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C63" s="8" t="n">
-        <v>54.02</v>
+        <v>64.27</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>2027</v>
+        <v>2023</v>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Euro/TL (ortalama)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C64" s="8" t="n">
-        <v>64.69</v>
+        <v>64.77</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C65" s="8" t="n">
-        <v>79.89</v>
+        <v>44.38</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>2022</v>
+        <v>2025</v>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C66" s="8" t="n">
-        <v>97.72</v>
+        <v>30.89</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>2023</v>
+        <v>2026</v>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>TUFE (yil sonu) (%)</t>
         </is>
       </c>
       <c r="C67" s="8" t="n">
-        <v>44.22</v>
+        <v>29.68</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>2024</v>
+        <v>2021</v>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C68" s="8" t="n">
-        <v>28.52</v>
+        <v>-7.2</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C69" s="8" t="n">
-        <v>27.67</v>
+        <v>-48.8</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C70" s="8" t="n">
-        <v>29.52</v>
+        <v>-44</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n">
-        <v>2027</v>
+        <v>2024</v>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>UFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C71" s="8" t="n">
-        <v>20.37</v>
+        <v>-9.800000000000001</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C72" s="8" t="n">
-        <v>36.08</v>
+        <v>-24</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C73" s="8" t="n">
-        <v>64.27</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>64.77</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>2024</v>
+        <v>2022</v>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C75" s="8" t="n">
-        <v>44.38</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C76" s="8" t="n">
-        <v>30.89</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C77" s="8" t="n">
-        <v>29.68</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>2027</v>
+        <v>2025</v>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>TUFE (yil sonu) (%)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C78" s="8" t="n">
-        <v>22.98</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>2021</v>
+        <v>2026</v>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Cari Islemler Dengesi / GSYH (%)</t>
         </is>
       </c>
       <c r="C79" s="8" t="n">
-        <v>-7.2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C80" s="8" t="n">
-        <v>-48.8</v>
+        <v>225</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C81" s="8" t="n">
-        <v>-44</v>
+        <v>254</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C82" s="8" t="n">
-        <v>-9.800000000000001</v>
+        <v>256</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C83" s="8" t="n">
-        <v>-24</v>
+        <v>262</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>-55</v>
+        <v>273</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi (milyar ABD $)</t>
+          <t>Ihracat (fob, milyar ABD $)</t>
         </is>
       </c>
       <c r="C85" s="8" t="n">
-        <v>-41</v>
+        <v>280</v>
       </c>
     </row>
     <row r="86">
@@ -2723,11 +2723,11 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C86" s="8" t="n">
-        <v>-0.9</v>
+        <v>271</v>
       </c>
     </row>
     <row r="87">
@@ -2736,11 +2736,11 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C87" s="8" t="n">
-        <v>-5.3</v>
+        <v>364</v>
       </c>
     </row>
     <row r="88">
@@ -2749,11 +2749,11 @@
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>-3.8</v>
+        <v>362</v>
       </c>
     </row>
     <row r="89">
@@ -2762,11 +2762,11 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C89" s="8" t="n">
-        <v>-0.7</v>
+        <v>344</v>
       </c>
     </row>
     <row r="90">
@@ -2775,11 +2775,11 @@
       </c>
       <c r="B90" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>-1.5</v>
+        <v>366</v>
       </c>
     </row>
     <row r="91">
@@ -2788,388 +2788,167 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Ithalat (cif, milyar ABD $)</t>
         </is>
       </c>
       <c r="C91" s="8" t="n">
-        <v>-3</v>
+        <v>400</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>2027</v>
+        <v>2021</v>
       </c>
       <c r="B92" s="8" t="inlineStr">
         <is>
-          <t>Cari Islemler Dengesi / GSYH (%)</t>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>-2</v>
+        <v>-46</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>225</v>
+        <v>-110</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B94" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
-        <v>254</v>
+        <v>-106</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B95" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>256</v>
+        <v>-82</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="8" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B96" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>262</v>
+        <v>-92</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B97" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>273</v>
+        <v>-120</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="8" t="n">
-        <v>2026</v>
+        <v>2021</v>
       </c>
       <c r="B98" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>280</v>
+        <v>71</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="n">
-        <v>2027</v>
+        <v>2022</v>
       </c>
       <c r="B99" s="8" t="inlineStr">
         <is>
-          <t>Ihracat (fob, milyar ABD $)</t>
+          <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>289</v>
+        <v>99</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="8" t="n">
-        <v>2021</v>
+        <v>2023</v>
       </c>
       <c r="B100" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>271</v>
+        <v>82</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="n">
-        <v>2022</v>
+        <v>2024</v>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>364</v>
+        <v>81</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="8" t="n">
-        <v>2023</v>
+        <v>2025</v>
       </c>
       <c r="B102" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>362</v>
+        <v>69</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
+          <t>Brent Petrol (ABD$/varil)</t>
         </is>
       </c>
       <c r="C103" s="8" t="n">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="8" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B104" s="8" t="inlineStr">
-        <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C104" s="8" t="n">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B105" s="8" t="inlineStr">
-        <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C105" s="8" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B106" s="8" t="inlineStr">
-        <is>
-          <t>Ithalat (cif, milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C106" s="8" t="n">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B107" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C107" s="8" t="n">
-        <v>-46</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="8" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B108" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="n">
-        <v>-110</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="8" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B109" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C109" s="8" t="n">
-        <v>-106</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B110" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C110" s="8" t="n">
-        <v>-82</v>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="8" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B111" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C111" s="8" t="n">
-        <v>-92</v>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B112" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C112" s="8" t="n">
-        <v>-120</v>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="8" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B113" s="8" t="inlineStr">
-        <is>
-          <t>Dis Ticaret Dengesi (milyar ABD $)</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="n">
-        <v>-91</v>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="8" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B114" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C114" s="8" t="n">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="8" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B115" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C115" s="8" t="n">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="8" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B116" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C116" s="8" t="n">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="8" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B117" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="n">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="8" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B118" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="n">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B119" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C119" s="8" t="n">
         <v>88</v>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="8" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B120" s="8" t="inlineStr">
-        <is>
-          <t>Brent Petrol (ABD$/varil)</t>
-        </is>
-      </c>
-      <c r="C120" s="8" t="n">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sayfa 3-4: RTG hatali fiyat duzeltmesi + kirik eksen; haftalik veri guncellemesi
- Fon Brosur'de RTG 19.10.2026 fiyati 1,636 yazilmisti (TEFAS: 5,5109);
  kaynak duzeltildi, fon getirileri / performans ozeti / RTG fiyat serisi
  yeniden uretildi. RTG Yillik -57,8% -> +42,2%, YBB -59,8% -> +35,3%.
- FonlarPerformansBarGrafik: -12%'nin altindaki barlar kirik eksenle
  ("//") gosteriliyor, etiket gercek degeri yaziyor; negatif etiketler
  barin solunda.
- Bekleyen haftalik veri guncellemesi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veri_Kaynagi.xlsx
+++ b/Veri_Kaynagi.xlsx
@@ -1466,7 +1466,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>12374</v>
+        <v>12251</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>11000</v>
@@ -1490,7 +1490,7 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>49.17</v>
+        <v>49.4</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>53</v>
@@ -1514,7 +1514,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>55.16</v>
+        <v>55.57</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>60.5</v>
@@ -1538,7 +1538,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7723</v>
+        <v>7812</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>7000</v>
@@ -1562,7 +1562,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>6272</v>
+        <v>6167</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>5800</v>
@@ -3036,7 +3036,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -3045,7 +3045,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>247.8</v>
+        <v>247.33</v>
       </c>
     </row>
     <row r="6">
@@ -3392,7 +3392,7 @@
         <v>2026</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4397,7 +4397,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
@@ -5113,7 +5113,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22.6</v>
+        <v>19.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5131,7 +5131,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>10.4</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26.9</v>
+        <v>21.8</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>32.9</v>
+        <v>27.6</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5185,7 +5185,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.2</v>
+        <v>12.9</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5203,7 +5203,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>37</v>
+        <v>36.3</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5221,7 +5221,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>30.6</v>
+        <v>27.6</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5239,7 +5239,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>49.2</v>
+        <v>49.1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5257,7 +5257,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>43</v>
+        <v>42.8</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5275,7 +5275,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5293,7 +5293,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>52.5</v>
+        <v>42.2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.2</v>
+        <v>15.2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>-3.2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>19.9</v>
+        <v>14.8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>34.1</v>
+        <v>35.3</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>19.9</v>
+        <v>20.7</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>18</v>
+        <v>18.3</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>16.9</v>
+        <v>12.8</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8.4</v>
+        <v>2.9</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5552,7 +5552,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25.3</v>
+        <v>19.1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>13.4</v>
+        <v>7.1</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5588,7 +5588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>13.2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5606,7 +5606,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22.9</v>
+        <v>21.5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -5624,7 +5624,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>45.8</v>
+        <v>35.3</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -5642,7 +5642,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.5</v>
+        <v>5.6</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -5660,7 +5660,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>29.2</v>
+        <v>24.5</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -5678,7 +5678,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>27.6</v>
+        <v>24.1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>33.6</v>
+        <v>34.5</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13.1</v>
+        <v>14.1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-1.4</v>
+        <v>-1</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -5768,7 +5768,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>26.6</v>
+        <v>26.3</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -5786,7 +5786,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>14.7</v>
+        <v>15.2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -5804,7 +5804,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>35.6</v>
+        <v>36.6</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -5822,7 +5822,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>30.2</v>
+        <v>31.1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -6791,7 +6791,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6808,13 +6808,13 @@
         <v>3.2</v>
       </c>
       <c r="E2" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6828,16 +6828,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6851,16 +6851,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="E4" t="n">
-        <v>21.6</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6874,16 +6874,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>43</v>
+        <v>42.8</v>
       </c>
       <c r="E5" t="n">
-        <v>45.2</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -6897,16 +6897,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>30.2</v>
+        <v>31.1</v>
       </c>
       <c r="E6" t="n">
-        <v>32.6</v>
+        <v>33.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6920,16 +6920,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-5.9</v>
+        <v>-2.6</v>
       </c>
       <c r="E7" t="n">
-        <v>-15.2</v>
+        <v>-10.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6943,16 +6943,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1.3</v>
+        <v>-1.4</v>
       </c>
       <c r="E8" t="n">
-        <v>-14.1</v>
+        <v>-16.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6966,16 +6966,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8.300000000000001</v>
+        <v>-0.9</v>
       </c>
       <c r="E9" t="n">
-        <v>-4.5</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6989,16 +6989,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>30.6</v>
+        <v>27.6</v>
       </c>
       <c r="E10" t="n">
-        <v>16.2</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -7012,16 +7012,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>27.6</v>
+        <v>24.1</v>
       </c>
       <c r="E11" t="n">
-        <v>10.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -7035,16 +7035,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-8.1</v>
+        <v>-6.2</v>
       </c>
       <c r="E12" t="n">
-        <v>-11.7</v>
+        <v>-8.300000000000001</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -7058,16 +7058,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-1.3</v>
+        <v>-5.5</v>
       </c>
       <c r="E13" t="n">
-        <v>-4.9</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -7081,16 +7081,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>-1.4</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -7104,16 +7104,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>28.2</v>
+        <v>28.4</v>
       </c>
       <c r="E15" t="n">
-        <v>26.8</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -7127,16 +7127,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>22.9</v>
+        <v>21.5</v>
       </c>
       <c r="E16" t="n">
-        <v>19.6</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -7150,16 +7150,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.8</v>
+        <v>-1.6</v>
       </c>
       <c r="E17" t="n">
-        <v>-10.4</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -7173,16 +7173,16 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.4</v>
+        <v>-0.9</v>
       </c>
       <c r="E18" t="n">
-        <v>-10.7</v>
+        <v>-14.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -7196,16 +7196,16 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>47</v>
+        <v>27.9</v>
       </c>
       <c r="E19" t="n">
-        <v>15.7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -7219,16 +7219,16 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>52.5</v>
+        <v>42.2</v>
       </c>
       <c r="E20" t="n">
-        <v>11.9</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -7242,16 +7242,16 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>45.8</v>
+        <v>35.3</v>
       </c>
       <c r="E21" t="n">
-        <v>17.3</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -7265,16 +7265,16 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-5.6</v>
+        <v>-2</v>
       </c>
       <c r="E22" t="n">
-        <v>-14.2</v>
+        <v>-10.8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7288,16 +7288,16 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>-2.5</v>
+        <v>-0.1</v>
       </c>
       <c r="E23" t="n">
-        <v>-19.6</v>
+        <v>-18.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7311,16 +7311,16 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.2</v>
+        <v>-4.8</v>
       </c>
       <c r="E24" t="n">
-        <v>-9.1</v>
+        <v>-15.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -7334,16 +7334,16 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>12.2</v>
+        <v>15.2</v>
       </c>
       <c r="E25" t="n">
-        <v>1.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -7357,16 +7357,16 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>12</v>
+        <v>13.2</v>
       </c>
       <c r="E26" t="n">
-        <v>3.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -7380,16 +7380,16 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>-13.5</v>
+        <v>-9.5</v>
       </c>
       <c r="E27" t="n">
-        <v>-17.5</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -7403,16 +7403,16 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>-4.4</v>
+        <v>-6.2</v>
       </c>
       <c r="E28" t="n">
-        <v>-10.3</v>
+        <v>-12.4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7426,16 +7426,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-1.4</v>
+        <v>-14</v>
       </c>
       <c r="E29" t="n">
-        <v>-12.7</v>
+        <v>-25.9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7449,16 +7449,16 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>-3.2</v>
       </c>
       <c r="E30" t="n">
-        <v>-3.3</v>
+        <v>-14.6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7472,16 +7472,16 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>13.4</v>
+        <v>7.1</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7495,16 +7495,16 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>-9.1</v>
+        <v>-6.8</v>
       </c>
       <c r="E32" t="n">
-        <v>-6.1</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7518,16 +7518,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>-4.7</v>
+        <v>-11.3</v>
       </c>
       <c r="E33" t="n">
-        <v>4.7</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7541,16 +7541,16 @@
         </is>
       </c>
       <c r="D34" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="E34" t="n">
         <v>-1.2</v>
-      </c>
-      <c r="E34" t="n">
-        <v>11.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7564,16 +7564,16 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>15</v>
+        <v>10.4</v>
       </c>
       <c r="E35" t="n">
-        <v>37</v>
+        <v>36.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7587,16 +7587,16 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8.4</v>
+        <v>2.9</v>
       </c>
       <c r="E36" t="n">
-        <v>29.2</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7610,16 +7610,16 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4336.8</v>
+        <v>4115.2</v>
       </c>
       <c r="E37" t="n">
-        <v>5145.8</v>
+        <v>4952.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7633,16 +7633,16 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-5.4</v>
+        <v>-2.4</v>
       </c>
       <c r="E38" t="n">
-        <v>-15.2</v>
+        <v>-10.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7656,16 +7656,16 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-0.1</v>
+        <v>-3.6</v>
       </c>
       <c r="E39" t="n">
-        <v>-14.1</v>
+        <v>-16.4</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7679,16 +7679,16 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5.5</v>
+        <v>-6</v>
       </c>
       <c r="E40" t="n">
-        <v>-4.5</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7702,16 +7702,16 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>22.6</v>
+        <v>19.5</v>
       </c>
       <c r="E41" t="n">
-        <v>16.2</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7725,16 +7725,16 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>16.9</v>
+        <v>12.8</v>
       </c>
       <c r="E42" t="n">
-        <v>10.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7748,16 +7748,16 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5979.8</v>
+        <v>5768.4</v>
       </c>
       <c r="E43" t="n">
-        <v>2364.5</v>
+        <v>2255.9</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7771,16 +7771,16 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>72.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="E44" t="n">
-        <v>54.7</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7794,16 +7794,16 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1223</v>
+        <v>1159.4</v>
       </c>
       <c r="E45" t="n">
-        <v>893.4</v>
+        <v>841.8</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7817,16 +7817,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>-9.6</v>
+        <v>-5.6</v>
       </c>
       <c r="E46" t="n">
-        <v>-21.7</v>
+        <v>-17.3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7840,16 +7840,16 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-3.8</v>
+        <v>-11.3</v>
       </c>
       <c r="E47" t="n">
-        <v>-14.4</v>
+        <v>-23.4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7863,16 +7863,16 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>11.1</v>
+        <v>-3.1</v>
       </c>
       <c r="E48" t="n">
-        <v>-3.1</v>
+        <v>-15.7</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7886,16 +7886,16 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>32.9</v>
+        <v>27.6</v>
       </c>
       <c r="E49" t="n">
-        <v>17.2</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7909,16 +7909,16 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>25.3</v>
+        <v>19.1</v>
       </c>
       <c r="E50" t="n">
-        <v>18</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7932,16 +7932,16 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>-3</v>
+        <v>-1.9</v>
       </c>
       <c r="E51" t="n">
-        <v>-3.7</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7955,16 +7955,16 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>6.9</v>
+        <v>8.5</v>
       </c>
       <c r="E52" t="n">
-        <v>6.7</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7978,16 +7978,16 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>-2</v>
+        <v>-3.6</v>
       </c>
       <c r="E53" t="n">
-        <v>-0.8</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -8001,16 +8001,16 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>19.9</v>
+        <v>14.8</v>
       </c>
       <c r="E54" t="n">
-        <v>25.2</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -8027,13 +8027,13 @@
         <v>6</v>
       </c>
       <c r="E55" t="n">
-        <v>9</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -8053,7 +8053,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -8067,13 +8067,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8.800000000000001</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -8087,13 +8087,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>26.8</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -8107,13 +8107,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34.1</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -8127,13 +8127,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>26.6</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -8156,7 +8156,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -8170,16 +8170,16 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>10.1</v>
+        <v>9.9</v>
       </c>
       <c r="E62" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -8193,7 +8193,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="E63" t="n">
         <v>21.3</v>
@@ -8202,7 +8202,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -8216,16 +8216,16 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>49.2</v>
+        <v>49.1</v>
       </c>
       <c r="E64" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -8239,16 +8239,16 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>35.6</v>
+        <v>36.6</v>
       </c>
       <c r="E65" t="n">
-        <v>33.6</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -8262,16 +8262,16 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>-0.9</v>
+        <v>0.7</v>
       </c>
       <c r="E66" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -8285,7 +8285,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="E67" t="n">
         <v>0.7</v>
@@ -8294,7 +8294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>10.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E68" t="n">
         <v>1.3</v>
@@ -8317,7 +8317,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>19.9</v>
+        <v>20.7</v>
       </c>
       <c r="E69" t="n">
         <v>2.2</v>
@@ -8340,7 +8340,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -8354,7 +8354,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>13.1</v>
+        <v>14.1</v>
       </c>
       <c r="E70" t="n">
         <v>1.8</v>
@@ -8363,7 +8363,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -8383,7 +8383,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -8397,13 +8397,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>9.9</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21.7</v>
+        <v>21.6</v>
       </c>
     </row>
   </sheetData>
@@ -8480,7 +8480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8499,13 +8499,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8524,13 +8524,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8549,13 +8549,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10.3</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8574,13 +8574,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>18</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8599,13 +8599,13 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>14.7</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8630,7 +8630,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8649,13 +8649,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8680,7 +8680,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8699,13 +8699,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8724,13 +8724,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>33.6</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8749,13 +8749,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>-7.9</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8774,13 +8774,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -8824,13 +8824,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>31.2</v>
+        <v>38.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -8849,13 +8849,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>27.8</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -8874,13 +8874,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>-18.9</v>
+        <v>-19.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -8899,13 +8899,13 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>-22.8</v>
+        <v>-33</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -8924,13 +8924,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>-7.9</v>
+        <v>-21.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -8949,13 +8949,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>18.6</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8974,13 +8974,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>4.5</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -8999,13 +8999,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>6.4</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9024,13 +9024,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>12.8</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9049,13 +9049,13 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>42.2</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9074,13 +9074,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>28.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9099,13 +9099,13 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>33.4</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -9124,13 +9124,13 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>-41.6</v>
+        <v>-34.6</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -9149,13 +9149,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>-54.3</v>
+        <v>-60.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -9174,13 +9174,13 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>-33.5</v>
+        <v>-42.8</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -9199,13 +9199,13 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>-18.8</v>
+        <v>-26.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -9224,13 +9224,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>-12.6</v>
+        <v>-21.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -9249,13 +9249,13 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>3.15</v>
+        <v>3.13</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -9274,13 +9274,13 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>10.43</v>
+        <v>10.35</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9299,13 +9299,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>22.37</v>
+        <v>22.29</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -9324,13 +9324,13 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>49.21</v>
+        <v>49.06</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -9349,7 +9349,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>36.05</v>
+        <v>37.02</v>
       </c>
     </row>
   </sheetData>
@@ -9463,7 +9463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9497,7 +9497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9511,13 +9511,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10.18</v>
+        <v>10.45</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9531,13 +9531,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8.93</v>
+        <v>9.41</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9551,13 +9551,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.87</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9571,13 +9571,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.18</v>
+        <v>4.84</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9587,17 +9587,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9607,17 +9607,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.8100000000000001</v>
+        <v>15.87</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9627,17 +9627,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Takasbank Para Piyasası</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>17.25</v>
+        <v>30.13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9647,17 +9647,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>32.16</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9667,17 +9667,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.6899999999999999</v>
+        <v>23.42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9687,17 +9687,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24.24</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -9711,13 +9711,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10.55</v>
+        <v>10.66</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -9731,13 +9731,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>72.81999999999999</v>
+        <v>72.59</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9751,13 +9751,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>16.63</v>
+        <v>16.75</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9771,13 +9771,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>88.89</v>
+        <v>83.52</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9791,13 +9791,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3.25</v>
+        <v>6.33</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9811,13 +9811,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7.86</v>
+        <v>10.15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9831,13 +9831,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>9.390000000000001</v>
+        <v>9.380000000000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9851,13 +9851,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4.23</v>
+        <v>4.24</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9871,13 +9871,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>59.6</v>
+        <v>54.71</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9891,13 +9891,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>26.78</v>
+        <v>31.67</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9907,17 +9907,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Kamu Dış Borçlanma Araçları</t>
+          <t>Vadeli Mevduat (Döviz)</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>84.69</v>
+        <v>14.72</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9927,17 +9927,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (Döviz)</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>12.91</v>
+        <v>3.08</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9947,17 +9947,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Özel Sektör Dış Borçlanma Araçları</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2.4</v>
+        <v>82.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -9971,13 +9971,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>85.73999999999999</v>
+        <v>87.27</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -9991,13 +9991,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.33</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10011,13 +10011,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3.83</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10031,13 +10031,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.31</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10051,13 +10051,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5.79</v>
+        <v>6.53</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10077,7 +10077,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10087,17 +10087,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.24</v>
+        <v>4.43</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10107,17 +10107,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Özel Sektör Tahvili</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.88</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -10127,17 +10127,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Takasbank Para Piyasası</t>
+          <t>Özel Sektör Tahvili</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>17.82</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10147,17 +10147,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ters Repo</t>
+          <t>Takasbank Para Piyasası</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>43.63</v>
+        <v>15.03</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10167,17 +10167,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Varlığa Dayalı Menkul Kıymet</t>
+          <t>Ters Repo</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.54</v>
+        <v>40.79</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -10187,37 +10187,37 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Vadeli Mevduat (TL)</t>
+          <t>Varlığa Dayalı Menkul Kıymet</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>35.25</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JET</t>
+          <t>DGH</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Vadeli Mevduat (TL)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>22.45</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -10227,17 +10227,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.49</v>
+        <v>21.43</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -10247,17 +10247,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>68.48999999999999</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -10267,37 +10267,37 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8.57</v>
+        <v>68.86</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PKF</t>
+          <t>JET</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>9.41</v>
+        <v>8.06</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -10307,17 +10307,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3.99</v>
+        <v>9.710000000000001</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10327,17 +10327,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Kıymetli Maden</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>82.7</v>
+        <v>5.18</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10347,37 +10347,37 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Kıymetli Maden</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3.9</v>
+        <v>81.62</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PKP</t>
+          <t>PKF</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BİST Vadeli İşlem (Satım)</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>53.49</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10387,17 +10387,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Katılma Hesabı (TL)</t>
+          <t>BİST Vadeli İşlem (Satım)</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>24.94</v>
+        <v>58.31</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10407,37 +10407,37 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Özel Sektör Kira Sertifikası</t>
+          <t>Katılma Hesabı (TL)</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>21.57</v>
+        <v>25.21</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RTG</t>
+          <t>PKP</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Özel Sektör Kira Sertifikası</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>19.17</v>
+        <v>16.48</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -10447,17 +10447,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.62</v>
+        <v>19.62</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -10467,17 +10467,17 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>68.75</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10487,37 +10487,37 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>11.46</v>
+        <v>66.89</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>TLZ</t>
+          <t>RTG</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>89.62</v>
+        <v>11.66</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10527,37 +10527,37 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>10.38</v>
+        <v>89.19</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>URA</t>
+          <t>TLZ</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Finansman Bonosu</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2.35</v>
+        <v>10.81</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10567,17 +10567,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Finansman Bonosu</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>15.41</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10587,17 +10587,17 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.2</v>
+        <v>15.51</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10607,17 +10607,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>68.09999999999999</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10627,37 +10627,37 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Yatırım Fonu Katılma Payı</t>
+          <t>Yabancı Hisse Senedi</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>13.94</v>
+        <v>67.54000000000001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>YLC</t>
+          <t>URA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Yerli Hisse Senedi</t>
+          <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>29.43</v>
+        <v>14.36</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10667,17 +10667,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>VİOP Teminatı</t>
+          <t>Yerli Hisse Senedi</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.57</v>
+        <v>27.06</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -10687,17 +10687,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Yabancı Hisse Senedi</t>
+          <t>VİOP Teminatı</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>68.48999999999999</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -10707,11 +10707,31 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
+          <t>Yabancı Hisse Senedi</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>71.25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>YLC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
           <t>Yatırım Fonu Katılma Payı</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>0.51</v>
+      <c r="D63" t="n">
+        <v>0.48</v>
       </c>
     </row>
   </sheetData>
@@ -10821,25 +10841,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>22.6</v>
+        <v>19.5</v>
       </c>
       <c r="E2" t="n">
-        <v>72.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="F2" t="n">
-        <v>1223</v>
+        <v>1159.4</v>
       </c>
       <c r="G2" t="n">
-        <v>5979.8</v>
+        <v>5768.4</v>
       </c>
       <c r="H2" t="n">
-        <v>19.9</v>
+        <v>20.6</v>
       </c>
       <c r="I2" t="n">
-        <v>67.59999999999999</v>
+        <v>66</v>
       </c>
       <c r="J2" t="n">
-        <v>34.4</v>
+        <v>34</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -10864,25 +10884,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16.2</v>
+        <v>12.9</v>
       </c>
       <c r="E3" t="n">
-        <v>54.7</v>
+        <v>53.8</v>
       </c>
       <c r="F3" t="n">
-        <v>893.4</v>
+        <v>841.8</v>
       </c>
       <c r="G3" t="n">
-        <v>2364.5</v>
+        <v>2255.9</v>
       </c>
       <c r="H3" t="n">
-        <v>15.7</v>
+        <v>15.4</v>
       </c>
       <c r="I3" t="n">
-        <v>58.3</v>
+        <v>56.6</v>
       </c>
       <c r="J3" t="n">
-        <v>25.9</v>
+        <v>25.5</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -10907,22 +10927,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="E4" t="n">
-        <v>17.7</v>
+        <v>21.5</v>
       </c>
       <c r="F4" t="n">
-        <v>329.6</v>
+        <v>317.6</v>
       </c>
       <c r="G4" t="n">
-        <v>3615.3</v>
+        <v>3512.5</v>
       </c>
       <c r="H4" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="I4" t="n">
-        <v>9.300000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="J4" t="n">
         <v>8.5</v>
@@ -10950,25 +10970,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>25.3</v>
+        <v>22.1</v>
       </c>
       <c r="E5" t="n">
-        <v>82.2</v>
+        <v>85.2</v>
       </c>
       <c r="F5" t="n">
-        <v>1351</v>
+        <v>1281.3</v>
       </c>
       <c r="G5" t="n">
-        <v>7623.7</v>
+        <v>7355.1</v>
       </c>
       <c r="H5" t="n">
-        <v>22.1</v>
+        <v>22.8</v>
       </c>
       <c r="I5" t="n">
-        <v>70.7</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="J5" t="n">
-        <v>36.7</v>
+        <v>36.3</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -10993,25 +11013,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>16.2</v>
+        <v>12.9</v>
       </c>
       <c r="E6" t="n">
-        <v>54.7</v>
+        <v>53.8</v>
       </c>
       <c r="F6" t="n">
-        <v>893.4</v>
+        <v>841.8</v>
       </c>
       <c r="G6" t="n">
-        <v>2364.5</v>
+        <v>2255.9</v>
       </c>
       <c r="H6" t="n">
-        <v>15.7</v>
+        <v>15.4</v>
       </c>
       <c r="I6" t="n">
-        <v>58.3</v>
+        <v>56.6</v>
       </c>
       <c r="J6" t="n">
-        <v>25.9</v>
+        <v>25.5</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -11036,22 +11056,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="E7" t="n">
-        <v>27.5</v>
+        <v>31.4</v>
       </c>
       <c r="F7" t="n">
-        <v>457.6</v>
+        <v>439.5</v>
       </c>
       <c r="G7" t="n">
-        <v>5259.2</v>
+        <v>5099.2</v>
       </c>
       <c r="H7" t="n">
-        <v>6.4</v>
+        <v>7.4</v>
       </c>
       <c r="I7" t="n">
-        <v>12.4</v>
+        <v>12.5</v>
       </c>
       <c r="J7" t="n">
         <v>10.8</v>
@@ -11128,10 +11148,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19.9</v>
+        <v>20.6</v>
       </c>
       <c r="E2" t="n">
-        <v>15.7</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="3">
@@ -11151,10 +11171,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-1</v>
+        <v>-0.3</v>
       </c>
       <c r="E3" t="n">
-        <v>-4.5</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="4">
@@ -11174,10 +11194,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>67.59999999999999</v>
+        <v>66</v>
       </c>
       <c r="E4" t="n">
-        <v>58.3</v>
+        <v>56.6</v>
       </c>
     </row>
     <row r="5">
@@ -11197,10 +11217,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>19.1</v>
+        <v>18.6</v>
       </c>
       <c r="E5" t="n">
-        <v>12.5</v>
+        <v>11.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>